<commit_message>
Remove obsolete programme_update.xlsx file; update app.js to enhance overview layout functionality and state management; improve CSS for day-week styling and responsive design adjustments.
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -764,16 +764,6 @@
           <t>Experimental and theoretical studies of the properties of atomic nuclei</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Чувильский Ю. М.</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Yu. M. Tchuvil'sky</t>
-        </is>
-      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>blue</t>
@@ -806,16 +796,6 @@
           <t>Experimental and theoretical studies of nuclear reactions</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Сидорчук С. И.</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>S. I. Sidorchuk</t>
-        </is>
-      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>green</t>
@@ -848,16 +828,6 @@
           <t>Modern nuclear-physics methods, technologies and facilities</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Жеребчевский В. И.</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>V. I. Zherebchevsky</t>
-        </is>
-      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>orange</t>
@@ -890,16 +860,6 @@
           <t>Relativistic nuclear physics, particle physics and high-energy physics</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Ким В. Т.</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>V. T. Kim</t>
-        </is>
-      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>red</t>
@@ -932,16 +892,6 @@
           <t>Physics of few-body systems</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Яковлев С. Л.</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>S. L. Yakovlev</t>
-        </is>
-      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>purple</t>
@@ -974,16 +924,6 @@
           <t>Nuclear astrophysics and neutrino physics</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Наумов В. А.</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>V. A. Naumov</t>
-        </is>
-      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>teal</t>
@@ -1014,16 +954,6 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>Nuclear medicine, radiation therapy and radioecology</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Черняев А. П.</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>A. P. Chernyaev</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -3702,7 +3632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M199"/>
+  <dimension ref="A1:N199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3753,35 +3683,40 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Название</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Длительность (мин)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Начало</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Тематика</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Примечание (RU)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Примечание (EN)</t>
         </is>
@@ -3813,12 +3748,12 @@
           <t>Эдуард Эрнстович</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>80 лет НИИЯФ МГУ</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3848,12 +3783,12 @@
           <t>Елена Александровна</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>70 лет ОИЯИ</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3883,15 +3818,15 @@
           <t>Ростислав Владимирович</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Quasimagic Nuclei and Pseudospin Symmetry</t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>30</v>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3923,15 +3858,15 @@
           <t>Richard</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>First results and plans of the BM@N experiment at NICA</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>30</v>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -3963,15 +3898,15 @@
           <t>Владимир Иосифович</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Ядерная физика и диагностика</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>30</v>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -4003,15 +3938,15 @@
           <t>Юрий Михайлович</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Восьминуклонные системы под ab initio микроскопом: спектры, кластеризация, распад и резонансные ядерные реакции</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>30</v>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4043,15 +3978,15 @@
           <t>Баярто Константинович</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Проект компактного многозадачного нейтринного детектора на основе галлий содержащих сцинтилляторов.</t>
         </is>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>30</v>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -4083,12 +4018,12 @@
           <t>Иван Сергеевич</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Производимые и поставляемые ООО «Гамматек» системы: (ОЧГ-, CZT-, сцинтилляционные) – спектрометры, альфа-спектрометры, а также ФЭУ, Si-ФЭУ и модули электроники для построения научного эксперимента</t>
         </is>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4118,12 +4053,12 @@
           <t>А. В.</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>Новые возможности отечественных диджитайзеров для задач ядерной физики</t>
         </is>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4153,12 +4088,12 @@
           <t>Михаил</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Делитель пучка СИ в геометрии Лауэ</t>
         </is>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4188,15 +4123,15 @@
           <t>Сергей Иванович</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Экспериментальные исследования ядерной структуры. Лаборатория ядерных реакций им. Г.Н. Флерова</t>
         </is>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>30</v>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -4228,15 +4163,15 @@
           <t>Дарья Максимовна</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Status and physics program of the NICA-MPD experiment at JINR</t>
         </is>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
         <v>30</v>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4268,15 +4203,15 @@
           <t>Виктор Тимофеевич</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Spin Physics Detector (SPD) at the NICA collider: status and outlooks</t>
         </is>
       </c>
-      <c r="H14" t="n">
+      <c r="I14" t="n">
         <v>30</v>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -4308,15 +4243,15 @@
           <t>Владимир Николаевич</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Эффекты нарушения изотопической симметрии в ядерных столкновениях на SPS и NICA</t>
         </is>
       </c>
-      <c r="H15" t="n">
+      <c r="I15" t="n">
         <v>30</v>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -4348,15 +4283,15 @@
           <t>Василий Вадимович</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Исследования спиновых эффектов на ядерных мишенях в эксперименте СПАСЧАРМ</t>
         </is>
       </c>
-      <c r="H16" t="n">
+      <c r="I16" t="n">
         <v>30</v>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -4388,15 +4323,15 @@
           <t>Олег Валерьевич</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>ARIADNA Program for Applied Research at NICA: Present Status and Outlook.</t>
         </is>
       </c>
-      <c r="H17" t="n">
+      <c r="I17" t="n">
         <v>30</v>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4428,15 +4363,15 @@
           <t>Людмила Дмитриевна</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Overview on progress in neutrino physics</t>
         </is>
       </c>
-      <c r="H18" t="n">
+      <c r="I18" t="n">
         <v>30</v>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -4468,15 +4403,15 @@
           <t>Александр Петрович</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Актуальные проблемы развития ядерно-физических технологий для медицины и промышленности</t>
         </is>
       </c>
-      <c r="H19" t="n">
+      <c r="I19" t="n">
         <v>30</v>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -4508,15 +4443,15 @@
           <t>Михаил Игоревич</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>Обобщенная теория конечных ферми-систем: формализм, анализ и оценки новых эффектов</t>
         </is>
       </c>
-      <c r="H20" t="n">
+      <c r="I20" t="n">
         <v>30</v>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4548,15 +4483,15 @@
           <t>Алексей Александрович</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>Physics opportunities for the fixed-target experiment at the Nuclotron with the SRC detector setup</t>
         </is>
       </c>
-      <c r="H21" t="n">
+      <c r="I21" t="n">
         <v>30</v>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4588,15 +4523,15 @@
           <t>Александр Игоревич</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>Изучение свойств тяжелых и сверхтяжелых ядер в ЛЯР ОИЯИ</t>
         </is>
       </c>
-      <c r="H22" t="n">
+      <c r="I22" t="n">
         <v>30</v>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4628,15 +4563,15 @@
           <t>Антон Александрович</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>Коллаборация FLAP: задачи и перспективы</t>
         </is>
       </c>
-      <c r="H23" t="n">
+      <c r="I23" t="n">
         <v>30</v>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -4668,15 +4603,15 @@
           <t>Эдуард Эрнстович</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>Проблемы и перспективы физики частиц</t>
         </is>
       </c>
-      <c r="H24" t="n">
+      <c r="I24" t="n">
         <v>30</v>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -4708,15 +4643,15 @@
           <t>Игорь Анатольевич</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>Probing nuclear structure with spectator nucleons from collisions of relativistic nuclei</t>
         </is>
       </c>
-      <c r="H25" t="n">
+      <c r="I25" t="n">
         <v>30</v>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -4748,15 +4683,15 @@
           <t>Олег Иванович</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>Few-body systems with singular (zero-range) interactions: Some aspects of correct formulation and related problems.</t>
         </is>
       </c>
-      <c r="H26" t="n">
+      <c r="I26" t="n">
         <v>30</v>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -4788,15 +4723,15 @@
           <t>Владимир Владимирович</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>Международный центр нейтронных исследований на базе реактора ПИК</t>
         </is>
       </c>
-      <c r="H27" t="n">
+      <c r="I27" t="n">
         <v>30</v>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -4828,15 +4763,15 @@
           <t>Валерий Валерьевич</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>Стенд для исследования световыхода органических сцинтилляторов: результаты эксперимента с генератором DT-нейтронов</t>
         </is>
       </c>
-      <c r="H28" t="n">
+      <c r="I28" t="n">
         <v>30</v>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -4868,15 +4803,15 @@
           <t>Владимир Васильевич</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>Эксперименты на пучках фотонов: проблемы и перспективы</t>
         </is>
       </c>
-      <c r="H29" t="n">
+      <c r="I29" t="n">
         <v>30</v>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -4908,15 +4843,15 @@
           <t>Валентин</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>Exotic E1 resonances in nuclei</t>
         </is>
       </c>
-      <c r="H30" t="n">
+      <c r="I30" t="n">
         <v>30</v>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4948,15 +4883,15 @@
           <t>Лариса Витальевна</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>Спонтанное и низкоэнергетическое вынужденное тройное деление ядер-актинидов: механизмы процесса и характеристики продуктов тройного деления</t>
         </is>
       </c>
-      <c r="H31" t="n">
+      <c r="I31" t="n">
         <v>30</v>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -4988,15 +4923,15 @@
           <t>Дмитрий Евгеньевич</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="H32" s="4" t="inlineStr">
         <is>
           <t>Механизмы формирования спинов и угловые распределения фрагментов деления: bending- и wriggling-корреляции</t>
         </is>
       </c>
-      <c r="H32" t="n">
+      <c r="I32" t="n">
         <v>30</v>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5028,15 +4963,15 @@
           <t>Максим Николаевич</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="H33" s="4" t="inlineStr">
         <is>
           <t>Нейтринный телескоп Baikal-GVD: статус и основные физические результаты</t>
         </is>
       </c>
-      <c r="H33" t="n">
+      <c r="I33" t="n">
         <v>30</v>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -5068,15 +5003,15 @@
           <t>Александр Сергеевич</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>JUNO experiment: status report and perspectives</t>
         </is>
       </c>
-      <c r="H34" t="n">
+      <c r="I34" t="n">
         <v>30</v>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -5108,15 +5043,15 @@
           <t>Павел Сергеевич</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>Nuclear data in Russia: current status and possible prospects</t>
         </is>
       </c>
-      <c r="H35" t="n">
+      <c r="I35" t="n">
         <v>30</v>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -5148,15 +5083,15 @@
           <t>Александр</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="H36" s="4" t="inlineStr">
         <is>
           <t>Description of backbending in even Pu nuclei</t>
         </is>
       </c>
-      <c r="H36" t="n">
+      <c r="I36" t="n">
         <v>30</v>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5188,15 +5123,15 @@
           <t>Алексей Александрович</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr">
+      <c r="H37" s="4" t="inlineStr">
         <is>
           <t>Программа исследований структуры нуклонов и атомных ядер методом активной мишени</t>
         </is>
       </c>
-      <c r="H37" t="n">
+      <c r="I37" t="n">
         <v>30</v>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5228,15 +5163,15 @@
           <t>Дмитрий Михайлович</t>
         </is>
       </c>
-      <c r="G38" s="4" t="inlineStr">
+      <c r="H38" s="4" t="inlineStr">
         <is>
           <t>Исследование реакций радиационного захвата протона на ядрах р- и sd-оболочки в рамках высокоточных оболочечных моделей</t>
         </is>
       </c>
-      <c r="H38" t="n">
+      <c r="I38" t="n">
         <v>30</v>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -5271,7 +5206,7 @@
           <t>НИИЯФ</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr">
+      <c r="H39" s="4" t="inlineStr">
         <is>
           <t>Properties of two-nucleon momentum distributions for A=6 nuclei found within three-cluster model</t>
         </is>
@@ -5306,7 +5241,7 @@
           <t>НИИЯФ</t>
         </is>
       </c>
-      <c r="G40" s="4" t="inlineStr">
+      <c r="H40" s="4" t="inlineStr">
         <is>
           <t>Остаточное нейтрон-протонное взаимодействие и локальные массовые соотношения</t>
         </is>
@@ -5341,7 +5276,7 @@
           <t>Эстония</t>
         </is>
       </c>
-      <c r="G41" s="4" t="inlineStr">
+      <c r="H41" s="4" t="inlineStr">
         <is>
           <t>Measuring te dependence of proton - neutron interaction on the ditance between them</t>
         </is>
@@ -5376,7 +5311,7 @@
           <t>ИЯИ</t>
         </is>
       </c>
-      <c r="G42" s="4" t="inlineStr">
+      <c r="H42" s="4" t="inlineStr">
         <is>
           <t>Ab initio no core shell model calculations of sd-shell nuclei</t>
         </is>
@@ -5411,7 +5346,7 @@
           <t>ИЯИ</t>
         </is>
       </c>
-      <c r="G43" s="4" t="inlineStr">
+      <c r="H43" s="4" t="inlineStr">
         <is>
           <t>Экспериментальная и расчетная зависимости коэффициента внутренней конверсии электрон-позитронной пары от угла их разлета при испускании ее из высоко возбужденного ядра 8Ве*</t>
         </is>
@@ -5446,7 +5381,7 @@
           <t>НИИЯФ</t>
         </is>
       </c>
-      <c r="G44" s="4" t="inlineStr">
+      <c r="H44" s="4" t="inlineStr">
         <is>
           <t>Расчет асимптотических нормировочных коэффициентов для нестабильных изотопов олова с нуклонным потенциалом дисперсионной оптической модели</t>
         </is>
@@ -5481,7 +5416,7 @@
           <t>ТОГУ</t>
         </is>
       </c>
-      <c r="G45" s="4" t="inlineStr">
+      <c r="H45" s="4" t="inlineStr">
         <is>
           <t>Neural Network Extrapolation of NCSM Results for the 17C Nuclear Spectrum</t>
         </is>
@@ -5516,7 +5451,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G46" s="4" t="inlineStr">
+      <c r="H46" s="4" t="inlineStr">
         <is>
           <t>Wigner’s SU(4) spin-isospin symmetry and MNT&amp;fragmentation nuclear reactions</t>
         </is>
@@ -5551,7 +5486,7 @@
           <t>КИ-ПИЯФ</t>
         </is>
       </c>
-      <c r="G47" s="4" t="inlineStr">
+      <c r="H47" s="4" t="inlineStr">
         <is>
           <t>Новый экспериментальный метод изучения кластерной структуры ядер с помощью активной мишени</t>
         </is>
@@ -5586,7 +5521,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G48" s="4" t="inlineStr">
+      <c r="H48" s="4" t="inlineStr">
         <is>
           <t>GEANT4-моделирование экспериментальной установки «Монумент». Выбор оптимальной толщины мишени 136BaCO3 в исследовании обычного мюонного захвата</t>
         </is>
@@ -5621,7 +5556,7 @@
           <t>ПИЯФ</t>
         </is>
       </c>
-      <c r="G49" s="4" t="inlineStr">
+      <c r="H49" s="4" t="inlineStr">
         <is>
           <t>Одночастичная структура изомерных состояний сферических ядер</t>
         </is>
@@ -5656,7 +5591,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G50" s="4" t="inlineStr">
+      <c r="H50" s="4" t="inlineStr">
         <is>
           <t>Исследование структуры ядер с квадруполь-октупольной деформацией</t>
         </is>
@@ -5691,7 +5626,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G51" s="4" t="inlineStr">
+      <c r="H51" s="4" t="inlineStr">
         <is>
           <t>Мюонный захват на ядре 136Ba</t>
         </is>
@@ -5726,7 +5661,7 @@
           <t>МИФИ</t>
         </is>
       </c>
-      <c r="G52" s="4" t="inlineStr">
+      <c r="H52" s="4" t="inlineStr">
         <is>
           <t>Проверка CVC-гипотезы и унитарности матрицы СКМ на основе анализа скорректированных значений Ft для сверхразрешённых β‑переходов</t>
         </is>
@@ -5761,7 +5696,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G53" s="4" t="inlineStr">
+      <c r="H53" s="4" t="inlineStr">
         <is>
           <t>The β-delayed γ-transitions of neutron-rich nuclei</t>
         </is>
@@ -5796,7 +5731,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G54" s="4" t="inlineStr">
+      <c r="H54" s="4" t="inlineStr">
         <is>
           <t>Fine structure in giant resonances</t>
         </is>
@@ -5831,7 +5766,7 @@
           <t>ВНИИЭФ</t>
         </is>
       </c>
-      <c r="G55" s="4" t="inlineStr">
+      <c r="H55" s="4" t="inlineStr">
         <is>
           <t>Фотоядерные реакции на природном молибдене при энергии тормозного излучения 25 МэВ</t>
         </is>
@@ -5866,7 +5801,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G56" s="4" t="inlineStr">
+      <c r="H56" s="4" t="inlineStr">
         <is>
           <t>Изоспиновое расщепление гигантского дипольного резонанса на средних и тяжелых ядрах</t>
         </is>
@@ -5901,7 +5836,7 @@
           <t>Узбекистан</t>
         </is>
       </c>
-      <c r="G57" s="4" t="inlineStr">
+      <c r="H57" s="4" t="inlineStr">
         <is>
           <t>Коэффициенты δ(Е2/М1) для переходов из вибрационных состояний в 182,184W</t>
         </is>
@@ -5936,7 +5871,7 @@
           <t>ТПУ (Томск</t>
         </is>
       </c>
-      <c r="G58" s="4" t="inlineStr">
+      <c r="H58" s="4" t="inlineStr">
         <is>
           <t>The method for verifying the enhancement of multipole transitions by vortex photons via activity measurement</t>
         </is>
@@ -5971,7 +5906,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G59" s="4" t="inlineStr">
+      <c r="H59" s="4" t="inlineStr">
         <is>
           <t>Gamma de-excitation of 90mZr isomer</t>
         </is>
@@ -6006,7 +5941,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G60" s="4" t="inlineStr">
+      <c r="H60" s="4" t="inlineStr">
         <is>
           <t>Skyrme-type energy density functional with surface-peaked effective mass</t>
         </is>
@@ -6041,7 +5976,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G61" s="4" t="inlineStr">
+      <c r="H61" s="4" t="inlineStr">
         <is>
           <t>Exploring the superheavy nuclei using 50Ti and 54Cr beams as the projectile</t>
         </is>
@@ -6076,7 +6011,7 @@
           <t>ВГУ</t>
         </is>
       </c>
-      <c r="G62" s="4" t="inlineStr">
+      <c r="H62" s="4" t="inlineStr">
         <is>
           <t>Устойчивость оболочечной структуры сверхтяжёлых ядер в деформированных потенциалах Нильсона и Вудса–Саксона</t>
         </is>
@@ -6111,7 +6046,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G63" s="4" t="inlineStr">
+      <c r="H63" s="4" t="inlineStr">
         <is>
           <t>Исследование структуры и изомерии ядер гольмия</t>
         </is>
@@ -6146,7 +6081,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G64" s="4" t="inlineStr">
+      <c r="H64" s="4" t="inlineStr">
         <is>
           <t>Эмпирическая систематика периодов полураспада спонтанного деления и альфа-распада тяжелых и сверхтяжелых ядер</t>
         </is>
@@ -6181,7 +6116,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G65" s="4" t="inlineStr">
+      <c r="H65" s="4" t="inlineStr">
         <is>
           <t>Transition densities of spin-dipole excitations in 208Pb</t>
         </is>
@@ -6216,7 +6151,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G66" s="4" t="inlineStr">
+      <c r="H66" s="4" t="inlineStr">
         <is>
           <t>Isotopic dependence of the fission threshold in nuclei with Z=114 and Z=120</t>
         </is>
@@ -6251,7 +6186,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G67" s="4" t="inlineStr">
+      <c r="H67" s="4" t="inlineStr">
         <is>
           <t>Анализ альфа-распадных цепочек элементов 119 и 120 в двухцентровой оболочечной модели: конкуренция незапрещённых и запрещённых переходов</t>
         </is>
@@ -6286,7 +6221,7 @@
           <t>НИЦ КИ</t>
         </is>
       </c>
-      <c r="G68" s="4" t="inlineStr">
+      <c r="H68" s="4" t="inlineStr">
         <is>
           <t>Анализ рассеяния дейтронов на ядре 13C в области энергий 13–18 МэВ: структура возбуждённых состояний и нейтронное гало</t>
         </is>
@@ -6321,7 +6256,7 @@
           <t>НИЦ КИ</t>
         </is>
       </c>
-      <c r="G69" s="4" t="inlineStr">
+      <c r="H69" s="4" t="inlineStr">
         <is>
           <t>Анализ реакции срыва 13C(d,t)12C в области энергий 13–18 мэв: определение асимптотических нормировочных коэффициентов и структуры состояний ядра 12C</t>
         </is>
@@ -6356,7 +6291,7 @@
           <t>ВНИИА</t>
         </is>
       </c>
-      <c r="G70" s="4" t="inlineStr">
+      <c r="H70" s="4" t="inlineStr">
         <is>
           <t>Полный и парциальные астрофизические S-факторы реакции 3He(d, p)4He в микроскопическом кластерном подходе</t>
         </is>
@@ -6391,7 +6326,7 @@
           <t>НИИЯФ</t>
         </is>
       </c>
-      <c r="G71" s="4" t="inlineStr">
+      <c r="H71" s="4" t="inlineStr">
         <is>
           <t>Ab initio description of scattering</t>
         </is>
@@ -6426,7 +6361,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G72" s="4" t="inlineStr">
+      <c r="H72" s="4" t="inlineStr">
         <is>
           <t>Multinucleon transfer reactions in 7Li, 12C,40Ar, 40,48Ca + 197Au</t>
         </is>
@@ -6461,7 +6396,7 @@
           <t>ТГУ(Томск)</t>
         </is>
       </c>
-      <c r="G73" s="4" t="inlineStr">
+      <c r="H73" s="4" t="inlineStr">
         <is>
           <t>Мультикластерная реализация задачи трёх тел на примере ядерных реакций с лёгкими ядрами</t>
         </is>
@@ -6496,7 +6431,7 @@
           <t>НИИЯФ</t>
         </is>
       </c>
-      <c r="G74" s="4" t="inlineStr">
+      <c r="H74" s="4" t="inlineStr">
         <is>
           <t>Учет кулоновской асимптотики в формализме осцилляторного представления теории рассеяния</t>
         </is>
@@ -6531,7 +6466,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G75" s="4" t="inlineStr">
+      <c r="H75" s="4" t="inlineStr">
         <is>
           <t>Excitation and decay of the Gamow-Teller resonance and its satellites in compaund nuclei</t>
         </is>
@@ -6566,7 +6501,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G76" s="4" t="inlineStr">
+      <c r="H76" s="4" t="inlineStr">
         <is>
           <t>Status of research on fissioning isomers in the fragments of binary fission of heavy nuclei</t>
         </is>
@@ -6601,7 +6536,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G77" s="4" t="inlineStr">
+      <c r="H77" s="4" t="inlineStr">
         <is>
           <t>Theoretical and experimental investigation on the optimization of accelerator driven subcritical reactors</t>
         </is>
@@ -6636,7 +6571,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G78" s="4" t="inlineStr">
+      <c r="H78" s="4" t="inlineStr">
         <is>
           <t>Время-проекционная камера для исследования свойств распада сверхтяжелых ядер</t>
         </is>
@@ -6671,7 +6606,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G79" s="4" t="inlineStr">
+      <c r="H79" s="4" t="inlineStr">
         <is>
           <t>Активная аргоновая защита в низкофоновых экспериментах по поиску двойного безнейтринного бета распада GERDA и LEGEND</t>
         </is>
@@ -6706,7 +6641,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G80" s="4" t="inlineStr">
+      <c r="H80" s="4" t="inlineStr">
         <is>
           <t>Comparative study of simulated and measured isotope production in target and HPGe detector in muon capture experiments</t>
         </is>
@@ -6741,7 +6676,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G81" s="4" t="inlineStr">
+      <c r="H81" s="4" t="inlineStr">
         <is>
           <t>Development of the evaluated cross sections database for (n,xγ)-type reactions</t>
         </is>
@@ -6776,7 +6711,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G82" s="4" t="inlineStr">
+      <c r="H82" s="4" t="inlineStr">
         <is>
           <t>Measurements of the gamma-ray emission cross sections and angular distributions from (n, xγ) reactions with 14.1 MeV neutrons</t>
         </is>
@@ -6811,7 +6746,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G83" s="4" t="inlineStr">
+      <c r="H83" s="4" t="inlineStr">
         <is>
           <t>Измерение выхода фотоядерной реакции (γ,p5n) на ядре висмута</t>
         </is>
@@ -6846,7 +6781,7 @@
           <t>МГУ</t>
         </is>
       </c>
-      <c r="G84" s="4" t="inlineStr">
+      <c r="H84" s="4" t="inlineStr">
         <is>
           <t>Фотоядерные реакции с вылетом протонов на изотопах эрбия</t>
         </is>
@@ -6881,7 +6816,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G85" s="4" t="inlineStr">
+      <c r="H85" s="4" t="inlineStr">
         <is>
           <t>Изоспиновое расщепление гигантского дипольного резонанса на средних и тяжелых ядрах</t>
         </is>
@@ -6916,7 +6851,7 @@
           <t>НИИЯФ</t>
         </is>
       </c>
-      <c r="G86" s="4" t="inlineStr">
+      <c r="H86" s="4" t="inlineStr">
         <is>
           <t>Особенности фоторасщепления изотопов рения 185,187Re</t>
         </is>
@@ -6951,7 +6886,7 @@
           <t>ВГУ</t>
         </is>
       </c>
-      <c r="G87" s="4" t="inlineStr">
+      <c r="H87" s="4" t="inlineStr">
         <is>
           <t>Определение вероятностей формирования предразрывных конфигураций в тройном делении ядер</t>
         </is>
@@ -6986,7 +6921,7 @@
           <t>ВГУ</t>
         </is>
       </c>
-      <c r="G88" s="4" t="inlineStr">
+      <c r="H88" s="4" t="inlineStr">
         <is>
           <t>Моменты инерции bending-моды и их влияние на спины фрагментов деления</t>
         </is>
@@ -7021,7 +6956,7 @@
           <t>Бангладеш</t>
         </is>
       </c>
-      <c r="G89" s="4" t="inlineStr">
+      <c r="H89" s="4" t="inlineStr">
         <is>
           <t>Potential description of alpha+197Au elastic scattering</t>
         </is>
@@ -7056,7 +6991,7 @@
           <t>ВНИИА</t>
         </is>
       </c>
-      <c r="G90" s="4" t="inlineStr">
+      <c r="H90" s="4" t="inlineStr">
         <is>
           <t>Описание дифференциальных сечений упругого рассеяния изотопов водорода в теории прямых ядерных реакций</t>
         </is>
@@ -7091,7 +7026,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G91" s="4" t="inlineStr">
+      <c r="H91" s="4" t="inlineStr">
         <is>
           <t>Исследование рассеяния 6He - 4He на фрагмент-сепараторе АКУЛИНА-2</t>
         </is>
@@ -7126,7 +7061,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G92" s="4" t="inlineStr">
+      <c r="H92" s="4" t="inlineStr">
         <is>
           <t>Experimental studies of 10B(7Li, 8Li)9B transfer reaction at 58 MeV</t>
         </is>
@@ -7161,7 +7096,7 @@
           <t>ИЯИ</t>
         </is>
       </c>
-      <c r="G93" s="4" t="inlineStr">
+      <c r="H93" s="4" t="inlineStr">
         <is>
           <t>Экспериментальный поиск аномалии при снятии возбуждения ядра 8Ве* с испусканием электрон-позитронной пары в реакции взаимодействия нейтронов с энергией свыше 20 МэВ с ядром 10В</t>
         </is>
@@ -7196,7 +7131,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G94" s="4" t="inlineStr">
+      <c r="H94" s="4" t="inlineStr">
         <is>
           <t>Изучение механизмов выбивания нейтрона в реакции 9Be(7Be, 6Be)X при промежуточной энергии</t>
         </is>
@@ -7231,7 +7166,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G95" s="4" t="inlineStr">
+      <c r="H95" s="4" t="inlineStr">
         <is>
           <t>Измерение угловых распределений распада 7He заселяемого в реакции 6He(d,p)</t>
         </is>
@@ -7266,7 +7201,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G96" s="4" t="inlineStr">
+      <c r="H96" s="4" t="inlineStr">
         <is>
           <t>Analytical approach to the generation of angular momentum in spontaneous fission fragments</t>
         </is>
@@ -7301,7 +7236,7 @@
           <t>МГУ</t>
         </is>
       </c>
-      <c r="G97" s="4" t="inlineStr">
+      <c r="H97" s="4" t="inlineStr">
         <is>
           <t>Исследование протон-индуцированных реакций на висмуте-209</t>
         </is>
@@ -7336,7 +7271,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G98" s="4" t="inlineStr">
+      <c r="H98" s="4" t="inlineStr">
         <is>
           <t>237Np+48Ca reaction and decay properties of 282Nh and descendant nuclei at DGFRS‑2</t>
         </is>
@@ -7371,7 +7306,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G99" s="4" t="inlineStr">
+      <c r="H99" s="4" t="inlineStr">
         <is>
           <t>Modeling of isotopic scaling and target ratio in transport statistical approach</t>
         </is>
@@ -7406,7 +7341,7 @@
           <t>ВГУ, ОИЯИ</t>
         </is>
       </c>
-      <c r="G100" s="4" t="inlineStr">
+      <c r="H100" s="4" t="inlineStr">
         <is>
           <t>Роль нейтронного избытка в механизмах передачи нуклонов в реакциях тяжелых ионов 40, 48Ca + 197Au</t>
         </is>
@@ -7441,7 +7376,7 @@
           <t>СПбГУ</t>
         </is>
       </c>
-      <c r="G101" s="4" t="inlineStr">
+      <c r="H101" s="4" t="inlineStr">
         <is>
           <t>Multi-agent modeling of collective dynamics in heavy nuclei fission</t>
         </is>
@@ -7476,7 +7411,7 @@
           <t>НИИЯФ</t>
         </is>
       </c>
-      <c r="G102" s="4" t="inlineStr">
+      <c r="H102" s="4" t="inlineStr">
         <is>
           <t>Neutron yield uncertainty calculations for (α, n) reactions using the NeuCBOT program</t>
         </is>
@@ -7511,7 +7446,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G103" s="4" t="inlineStr">
+      <c r="H103" s="4" t="inlineStr">
         <is>
           <t>Theoretical calculation of the angular anisotropy of gamma radiation on carbon, cromium and iron nuclei in inelastic neutron scattering</t>
         </is>
@@ -7546,7 +7481,7 @@
           <t>МГУ</t>
         </is>
       </c>
-      <c r="G104" s="4" t="inlineStr">
+      <c r="H104" s="4" t="inlineStr">
         <is>
           <t>Исследование эффекта наложения сигналов (pile-up) при регистрации ат-мосферных мюонов в нейтринном телескопе Baikal-GVD.</t>
         </is>
@@ -7581,7 +7516,7 @@
           <t>НИЦ КИ</t>
         </is>
       </c>
-      <c r="G105" s="4" t="inlineStr">
+      <c r="H105" s="4" t="inlineStr">
         <is>
           <t>Виртуальный генератор потока АТМОСФЕРНЫХ мюонов В варьируемом диапазоне энергий до 100 ТэВ</t>
         </is>
@@ -7616,7 +7551,7 @@
           <t>НИЦ КИ</t>
         </is>
       </c>
-      <c r="G106" s="4" t="inlineStr">
+      <c r="H106" s="4" t="inlineStr">
         <is>
           <t>Мюонная томография крупномасштабных объектов с применением компактных цилиндрических позиционно-чувствительных детекторов</t>
         </is>
@@ -7651,7 +7586,7 @@
           <t>ВНИИЭФ</t>
         </is>
       </c>
-      <c r="G107" s="4" t="inlineStr">
+      <c r="H107" s="4" t="inlineStr">
         <is>
           <t>Реконструкция плотности многокомпонентных объектов в протонной радиографии с использованием метода роя частиц и преобразования Абеля</t>
         </is>
@@ -7686,7 +7621,7 @@
           <t>ИЯФ Новосиб</t>
         </is>
       </c>
-      <c r="G108" s="4" t="inlineStr">
+      <c r="H108" s="4" t="inlineStr">
         <is>
           <t>Измерение ионизационных выходов ядер отдачи в аргоне</t>
         </is>
@@ -7721,7 +7656,7 @@
           <t>МИФИ</t>
         </is>
       </c>
-      <c r="G109" s="4" t="inlineStr">
+      <c r="H109" s="4" t="inlineStr">
         <is>
           <t>Development of machine learning tool for photon identification using the electromagnetic calorimeter at SPD detector</t>
         </is>
@@ -7756,7 +7691,7 @@
           <t>СПбГУ</t>
         </is>
       </c>
-      <c r="G110" s="4" t="inlineStr">
+      <c r="H110" s="4" t="inlineStr">
         <is>
           <t>Особенности изучения свойств пучков тяжёлых ионов высоких энергий</t>
         </is>
@@ -7791,7 +7726,7 @@
           <t>НИЦ КИ</t>
         </is>
       </c>
-      <c r="G111" s="4" t="inlineStr">
+      <c r="H111" s="4" t="inlineStr">
         <is>
           <t>Критический стенд «П»: современное состояние, особенности и роль исследований для развития технологии ВВЭР</t>
         </is>
@@ -7826,7 +7761,7 @@
           <t>ВНИИЭф</t>
         </is>
       </c>
-      <c r="G112" s="4" t="inlineStr">
+      <c r="H112" s="4" t="inlineStr">
         <is>
           <t>Результаты экспериментов с тепловыми трубами с цезиевым теплоносителем</t>
         </is>
@@ -7861,7 +7796,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G113" s="4" t="inlineStr">
+      <c r="H113" s="4" t="inlineStr">
         <is>
           <t>Низкофоновый детектор нейтронов на основе гелия-3</t>
         </is>
@@ -7896,7 +7831,7 @@
           <t>ВНИИА</t>
         </is>
       </c>
-      <c r="G114" s="4" t="inlineStr">
+      <c r="H114" s="4" t="inlineStr">
         <is>
           <t>Нейтрон-нейтронные методы дистанционного контроля с использованием меченых нейтронов</t>
         </is>
@@ -7931,7 +7866,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G115" s="4" t="inlineStr">
+      <c r="H115" s="4" t="inlineStr">
         <is>
           <t>Моделирование ионной оптики сепаратора STAR с помощью программы SHEMAT</t>
         </is>
@@ -7966,7 +7901,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G116" s="4" t="inlineStr">
+      <c r="H116" s="4" t="inlineStr">
         <is>
           <t>Криогенная газовая ячейка охлаждения ионов. Особенности конструкции, вакуумная система, система газового обеспечения, система охлаждения</t>
         </is>
@@ -8001,7 +7936,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G117" s="4" t="inlineStr">
+      <c r="H117" s="4" t="inlineStr">
         <is>
           <t>Измерение времени экстракции ионов из криогенной газовой ячейки охлаждения</t>
         </is>
@@ -8036,7 +7971,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G118" s="4" t="inlineStr">
+      <c r="H118" s="4" t="inlineStr">
         <is>
           <t>Нейтронные сцинтилляторы на основе кристалла ZnS(Ag)</t>
         </is>
@@ -8071,7 +8006,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G119" s="4" t="inlineStr">
+      <c r="H119" s="4" t="inlineStr">
         <is>
           <t>Физическая структура кросс-толка гамма-квантов в сферических многодетекторных сцинтилляционных системах</t>
         </is>
@@ -8106,7 +8041,7 @@
           <t>ИЯИ</t>
         </is>
       </c>
-      <c r="G120" s="4" t="inlineStr">
+      <c r="H120" s="4" t="inlineStr">
         <is>
           <t>Performance and light yield of CsI(pure) scintillation module prototypes at LN2 temperature</t>
         </is>
@@ -8141,7 +8076,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G121" s="4" t="inlineStr">
+      <c r="H121" s="4" t="inlineStr">
         <is>
           <t>Пласстмассовые сцинтилляторы с возможностью разделения частиц по форме импульса</t>
         </is>
@@ -8176,7 +8111,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G122" s="4" t="inlineStr">
+      <c r="H122" s="4" t="inlineStr">
         <is>
           <t>Исследование радиационной стойкости SiC- и Si-детекторов после облучения альфа-частицами</t>
         </is>
@@ -8211,7 +8146,7 @@
           <t>ПИЯФ</t>
         </is>
       </c>
-      <c r="G123" s="4" t="inlineStr">
+      <c r="H123" s="4" t="inlineStr">
         <is>
           <t>Average Spatial Resolution of Detector Layers of Four-Layer Position-Sensitive Detectors</t>
         </is>
@@ -8246,7 +8181,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G124" s="4" t="inlineStr">
+      <c r="H124" s="4" t="inlineStr">
         <is>
           <t>Применение диджитайзеров CAEN-ХХ42 для регистрации заряженных частиц</t>
         </is>
@@ -8281,7 +8216,7 @@
           <t>МГУ</t>
         </is>
       </c>
-      <c r="G125" s="4" t="inlineStr">
+      <c r="H125" s="4" t="inlineStr">
         <is>
           <t>Исследование распределения поглощённой дозы в полимерных материалах при облучении ускоренными электронами</t>
         </is>
@@ -8316,7 +8251,7 @@
           <t>СВКНИИ ДВО</t>
         </is>
       </c>
-      <c r="G126" s="4" t="inlineStr">
+      <c r="H126" s="4" t="inlineStr">
         <is>
           <t>Влияние 222Rn на расчёт радиоуглеродного возраста древесных углей</t>
         </is>
@@ -8351,7 +8286,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G127" s="4" t="inlineStr">
+      <c r="H127" s="4" t="inlineStr">
         <is>
           <t>Nd/ZnS-модифицированные квантовые точки CdZnSeS как нанокомпоненты сцинтилляционных сред для поиска безнейтринного двойного β-распада ¹⁵⁰Nd</t>
         </is>
@@ -8386,7 +8321,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G128" s="4" t="inlineStr">
+      <c r="H128" s="4" t="inlineStr">
         <is>
           <t>Results of ARFIM experiment setup for applied research of NOSU</t>
         </is>
@@ -8421,7 +8356,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G129" s="4" t="inlineStr">
+      <c r="H129" s="4" t="inlineStr">
         <is>
           <t>Neodymium-modified CdZnSeS/ZnS quantum dots: evolution of optical response and evidence limits for core/shell architecture</t>
         </is>
@@ -8451,7 +8386,7 @@
           <t>Анна Станиславовна</t>
         </is>
       </c>
-      <c r="G130" s="4" t="inlineStr">
+      <c r="H130" s="4" t="inlineStr">
         <is>
           <t>Перспективы применения сухой ионно-плазменной технологии дезактивации оборудования ЯЭУ из титановых сплавов</t>
         </is>
@@ -8486,7 +8421,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G131" s="4" t="inlineStr">
+      <c r="H131" s="4" t="inlineStr">
         <is>
           <t>Investigation of nuclear deformation influence on anisotropic flows in heavy-ion collisions at NICA energies</t>
         </is>
@@ -8521,7 +8456,7 @@
           <t>СПбГУ</t>
         </is>
       </c>
-      <c r="G132" s="4" t="inlineStr">
+      <c r="H132" s="4" t="inlineStr">
         <is>
           <t>Кумулятивные явления в области больших поперечных импульсов и их наблюдение в столкновениях ядер на коллайдере NICA</t>
         </is>
@@ -8556,7 +8491,7 @@
           <t>МГУ</t>
         </is>
       </c>
-      <c r="G133" s="4" t="inlineStr">
+      <c r="H133" s="4" t="inlineStr">
         <is>
           <t>Inclusive $J/\psi$ Production as a Probe of Gluon Dynamics at NICA</t>
         </is>
@@ -8591,7 +8526,7 @@
           <t>СПбГУ</t>
         </is>
       </c>
-      <c r="G134" s="4" t="inlineStr">
+      <c r="H134" s="4" t="inlineStr">
         <is>
           <t>Моделирование кумулятивных эффектов в столкновениях тяжелых ионов при энергиях коллайдера NICA</t>
         </is>
@@ -8626,7 +8561,7 @@
           <t>ИЯИ РАН</t>
         </is>
       </c>
-      <c r="G135" s="4" t="inlineStr">
+      <c r="H135" s="4" t="inlineStr">
         <is>
           <t>Методы определения центральности с использованием передних детекторов в эксперименте BM@N</t>
         </is>
@@ -8661,7 +8596,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G136" s="4" t="inlineStr">
+      <c r="H136" s="4" t="inlineStr">
         <is>
           <t>Λd сorrelation function in Xe+CsI collisions at 3.8 AGeV in the BM@N experiment</t>
         </is>
@@ -8696,7 +8631,7 @@
           <t>ИЯИ РАН</t>
         </is>
       </c>
-      <c r="G137" s="4" t="inlineStr">
+      <c r="H137" s="4" t="inlineStr">
         <is>
           <t>Measurement of double differential inclusive cross sections of forward neutron emission in the BM@N experiment</t>
         </is>
@@ -8731,7 +8666,7 @@
           <t>СПбГУ</t>
         </is>
       </c>
-      <c r="G138" s="4" t="inlineStr">
+      <c r="H138" s="4" t="inlineStr">
         <is>
           <t>Influence of colour string configurations on rapidity multiplicity correlations</t>
         </is>
@@ -8766,7 +8701,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G139" s="4" t="inlineStr">
+      <c r="H139" s="4" t="inlineStr">
         <is>
           <t>Эффективность и математические аналоги процедуры ИБП при вычислении интегралов Фейнмана</t>
         </is>
@@ -8801,7 +8736,7 @@
           <t>ДВФУ</t>
         </is>
       </c>
-      <c r="G140" s="4" t="inlineStr">
+      <c r="H140" s="4" t="inlineStr">
         <is>
           <t>Экранирование заряда в многокомпонентной аблелевой модели Хиггса</t>
         </is>
@@ -8836,7 +8771,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G141" s="4" t="inlineStr">
+      <c r="H141" s="4" t="inlineStr">
         <is>
           <t>Ядро 8Be и состояние Хойла в диссоциации релятивистских ядер</t>
         </is>
@@ -8871,7 +8806,7 @@
           <t>ИЯИ РАН</t>
         </is>
       </c>
-      <c r="G142" s="4" t="inlineStr">
+      <c r="H142" s="4" t="inlineStr">
         <is>
           <t>Dibaryon d*(2380) : prediction, detection, understanding</t>
         </is>
@@ -8906,7 +8841,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G143" s="4" t="inlineStr">
+      <c r="H143" s="4" t="inlineStr">
         <is>
           <t>pN spin amplitudes and spin observables of the pd →pd and dd →n+p+d processes</t>
         </is>
@@ -8941,7 +8876,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G144" s="4" t="inlineStr">
+      <c r="H144" s="4" t="inlineStr">
         <is>
           <t>Mass spectrum of noncharmed and charmed meson states at finite temperature in extended linear-sigma model</t>
         </is>
@@ -8976,7 +8911,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G145" s="4" t="inlineStr">
+      <c r="H145" s="4" t="inlineStr">
         <is>
           <t>Source velocity in collisions of 2.1 GeV and 3.6 GeV protons with gold target.</t>
         </is>
@@ -9011,7 +8946,7 @@
           <t>НИЦ КИ-ПИЯФ</t>
         </is>
       </c>
-      <c r="G146" s="4" t="inlineStr">
+      <c r="H146" s="4" t="inlineStr">
         <is>
           <t>Особенности измерения свойств резонансов в эксперименте MPD в Xe+W столкновениях при энергии 2,5 A*ГэВ</t>
         </is>
@@ -9046,7 +8981,7 @@
           <t>ИЯФ Новосиб</t>
         </is>
       </c>
-      <c r="G147" s="4" t="inlineStr">
+      <c r="H147" s="4" t="inlineStr">
         <is>
           <t>Pauli equation in spaces of constant curvature and extended Nikiforov-Uvarov method</t>
         </is>
@@ -9081,7 +9016,7 @@
           <t>СПбГУ</t>
         </is>
       </c>
-      <c r="G148" s="4" t="inlineStr">
+      <c r="H148" s="4" t="inlineStr">
         <is>
           <t>Минимизация объемных флуктуаций при поиске критической точки сильно взаимодействующей материи в релятивистских ядерных столкновениях</t>
         </is>
@@ -9116,7 +9051,7 @@
           <t>Tsinghua Univ., China</t>
         </is>
       </c>
-      <c r="G149" s="4" t="inlineStr">
+      <c r="H149" s="4" t="inlineStr">
         <is>
           <t>Heavy-flavor jet quenching in pre-equilibrium medium</t>
         </is>
@@ -9151,7 +9086,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G150" s="4" t="inlineStr">
+      <c r="H150" s="4" t="inlineStr">
         <is>
           <t>Overview of the STAR hot QCD results</t>
         </is>
@@ -9186,7 +9121,7 @@
           <t>СПбГУ</t>
         </is>
       </c>
-      <c r="G151" s="4" t="inlineStr">
+      <c r="H151" s="4" t="inlineStr">
         <is>
           <t>Исследование выходов заряженных адронов в рамках гидродинамического моделирования с применением голографического уравнения состояния</t>
         </is>
@@ -9221,7 +9156,7 @@
           <t>СПбГУ</t>
         </is>
       </c>
-      <c r="G152" s="4" t="inlineStr">
+      <c r="H152" s="4" t="inlineStr">
         <is>
           <t>Исследование нейросетевых подходов к оценке прицельного параметра в столкновениях тяжелых ионов на основе 4π информации о событии</t>
         </is>
@@ -9256,7 +9191,7 @@
           <t>НИЦ КИ-ПИЯФ</t>
         </is>
       </c>
-      <c r="G153" s="4" t="inlineStr">
+      <c r="H153" s="4" t="inlineStr">
         <is>
           <t>Неравновесный квантовый гидродинамический подход и эмиссия фрагментов в столкновениях тяжелых ионов промежуточных энергий</t>
         </is>
@@ -9291,7 +9226,7 @@
           <t>СПбГУ</t>
         </is>
       </c>
-      <c r="G154" s="4" t="inlineStr">
+      <c r="H154" s="4" t="inlineStr">
         <is>
           <t>Применение классического глауберовского подхода к описанию дейтрон-дейтронного взаимодействия</t>
         </is>
@@ -9326,7 +9261,7 @@
           <t>СПбГУ</t>
         </is>
       </c>
-      <c r="G155" s="4" t="inlineStr">
+      <c r="H155" s="4" t="inlineStr">
         <is>
           <t>О применении генераторов EPOS4, UrQMD, PHQMD и PYTHIA для анализа событий в физике сверхвысоких энергий</t>
         </is>
@@ -9361,7 +9296,7 @@
           <t>НИИЯФ МГУ</t>
         </is>
       </c>
-      <c r="G156" s="4" t="inlineStr">
+      <c r="H156" s="4" t="inlineStr">
         <is>
           <t>Моделирование влияния деформации ядер на азимутальную анизотропию частиц в генераторе событий HYDJET++</t>
         </is>
@@ -9396,7 +9331,7 @@
           <t>МИФИ</t>
         </is>
       </c>
-      <c r="G157" s="4" t="inlineStr">
+      <c r="H157" s="4" t="inlineStr">
         <is>
           <t>Analysis of charged and identified hadron spectra with Tsallis distributions in O+O, Kr+Kr, and Xe+Xe collisions at √sNN = 6 GeV using the UrQMD model</t>
         </is>
@@ -9431,7 +9366,7 @@
           <t>КИ ИФВЭ</t>
         </is>
       </c>
-      <c r="G158" s="4" t="inlineStr">
+      <c r="H158" s="4" t="inlineStr">
         <is>
           <t>Измерение выстроенности K*-(892)-мезонов, образованных в каон-ядерных и пион-ядерных взаимодействиях на ускорительном комплексе У-70</t>
         </is>
@@ -9466,7 +9401,7 @@
           <t>МИФИ</t>
         </is>
       </c>
-      <c r="G159" s="4" t="inlineStr">
+      <c r="H159" s="4" t="inlineStr">
         <is>
           <t>Поиск тринейтрона в реакциях поглощения остановившихся пионов ядрами 9Be</t>
         </is>
@@ -9501,7 +9436,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G160" s="4" t="inlineStr">
+      <c r="H160" s="4" t="inlineStr">
         <is>
           <t>Возможное существование синглетного дейтрона как дибарионного резонанса и проблема существования динейтрона</t>
         </is>
@@ -9536,7 +9471,7 @@
           <t>ТОГУ</t>
         </is>
       </c>
-      <c r="G161" s="4" t="inlineStr">
+      <c r="H161" s="4" t="inlineStr">
         <is>
           <t>Excited states of 6He nucleus in the SS-HORSE–NCSM approach</t>
         </is>
@@ -9571,7 +9506,7 @@
           <t>ТОГУ</t>
         </is>
       </c>
-      <c r="G162" s="4" t="inlineStr">
+      <c r="H162" s="4" t="inlineStr">
         <is>
           <t>Ионизация атомов протонным ударом в представлении параболических квазиштурмовских функций</t>
         </is>
@@ -9606,7 +9541,7 @@
           <t>ТОГУ</t>
         </is>
       </c>
-      <c r="G163" s="4" t="inlineStr">
+      <c r="H163" s="4" t="inlineStr">
         <is>
           <t>Атом водорода в поле лазерного импульса в представлении параболических волновых пакетов</t>
         </is>
@@ -9641,7 +9576,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G164" s="4" t="inlineStr">
+      <c r="H164" s="4" t="inlineStr">
         <is>
           <t>Van der Waals dimers of neon</t>
         </is>
@@ -9676,7 +9611,7 @@
           <t>НИИЯФ</t>
         </is>
       </c>
-      <c r="G165" s="4" t="inlineStr">
+      <c r="H165" s="4" t="inlineStr">
         <is>
           <t>Finding virtual states via wave-packet continuum discretization</t>
         </is>
@@ -9711,7 +9646,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G166" s="4" t="inlineStr">
+      <c r="H166" s="4" t="inlineStr">
         <is>
           <t>Resonances of a two-particle system on a 1D lattice</t>
         </is>
@@ -9746,7 +9681,7 @@
           <t>СПбГУ</t>
         </is>
       </c>
-      <c r="G167" s="4" t="inlineStr">
+      <c r="H167" s="4" t="inlineStr">
         <is>
           <t>3-3 рассеяние в системах трёх частиц с короткодействующими и кулоновскими взаимодействиями</t>
         </is>
@@ -9781,7 +9716,7 @@
           <t>ПИЯФ</t>
         </is>
       </c>
-      <c r="G168" s="4" t="inlineStr">
+      <c r="H168" s="4" t="inlineStr">
         <is>
           <t>Поиск тяжелого стерильного нейтрино в бета-распаде 144Pr</t>
         </is>
@@ -9816,7 +9751,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G169" s="4" t="inlineStr">
+      <c r="H169" s="4" t="inlineStr">
         <is>
           <t>Эффекты динамо и осцилляций в спектрах нейтрино сверхновых</t>
         </is>
@@ -9851,7 +9786,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G170" s="4" t="inlineStr">
+      <c r="H170" s="4" t="inlineStr">
         <is>
           <t>Эффекты намагниченности ядер во взрывном нуклеосинтезе</t>
         </is>
@@ -9886,7 +9821,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G171" s="4" t="inlineStr">
+      <c r="H171" s="4" t="inlineStr">
         <is>
           <t>Search for rare processes within the GeN experiment at Kalinin nuclear power plant</t>
         </is>
@@ -9921,7 +9856,7 @@
           <t>НИИЯФ</t>
         </is>
       </c>
-      <c r="G172" s="4" t="inlineStr">
+      <c r="H172" s="4" t="inlineStr">
         <is>
           <t>Precise reactor antineutrino spectrum measurement with TAO detector</t>
         </is>
@@ -9956,7 +9891,7 @@
           <t>НИИЯФ</t>
         </is>
       </c>
-      <c r="G173" s="4" t="inlineStr">
+      <c r="H173" s="4" t="inlineStr">
         <is>
           <t>Условия появления Λ-гиперонов в материи нейтронных звёзд в моделях среднего поля</t>
         </is>
@@ -9991,7 +9926,7 @@
           <t>Пакистан</t>
         </is>
       </c>
-      <c r="G174" s="4" t="inlineStr">
+      <c r="H174" s="4" t="inlineStr">
         <is>
           <t>Analysis of radiative capture of proton 11B (p, γ) 12C at low energy</t>
         </is>
@@ -10026,7 +9961,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G175" s="4" t="inlineStr">
+      <c r="H175" s="4" t="inlineStr">
         <is>
           <t>Characterization of the cosmic muon background in the NUGEN experiment</t>
         </is>
@@ -10056,7 +9991,7 @@
           <t>Василий Алексеевич</t>
         </is>
       </c>
-      <c r="G176" s="4" t="inlineStr">
+      <c r="H176" s="4" t="inlineStr">
         <is>
           <t>Подход к оптимизации распределения поглощенной дозы в биологическом объекте в лучевой терапии пучком ускоренных протонов</t>
         </is>
@@ -10091,7 +10026,7 @@
           <t>МГУ</t>
         </is>
       </c>
-      <c r="G177" s="4" t="inlineStr">
+      <c r="H177" s="4" t="inlineStr">
         <is>
           <t>Оценка рисков развития радиационно-индуцированных заболеваний при проведении лучевой терапии</t>
         </is>
@@ -10126,7 +10061,7 @@
           <t>НИЦ КИ ИФВЭ</t>
         </is>
       </c>
-      <c r="G178" s="4" t="inlineStr">
+      <c r="H178" s="4" t="inlineStr">
         <is>
           <t>Измерение сечения реакции 12C(12C,X)11C: особенности эксперимента и оценка неопределенностей</t>
         </is>
@@ -10161,7 +10096,7 @@
           <t>НИЦ КИ ИФВЭ</t>
         </is>
       </c>
-      <c r="G179" s="4" t="inlineStr">
+      <c r="H179" s="4" t="inlineStr">
         <is>
           <t>Реализация работы с данными КТ в системе планирования ионной лучевой терапии</t>
         </is>
@@ -10196,7 +10131,7 @@
           <t>СПбГУ</t>
         </is>
       </c>
-      <c r="G180" s="4" t="inlineStr">
+      <c r="H180" s="4" t="inlineStr">
         <is>
           <t>Трекинг, измерение энергии и получение диагностических изображений с использованием кремниевых пиксельных сенсоров</t>
         </is>
@@ -10231,7 +10166,7 @@
           <t>ИЯИ РАН</t>
         </is>
       </c>
-      <c r="G181" s="4" t="inlineStr">
+      <c r="H181" s="4" t="inlineStr">
         <is>
           <t>Реконструкция трёхмерного дозового рапсределения при облучении биологических объектов пучками протонов высокой интенсивности</t>
         </is>
@@ -10266,7 +10201,7 @@
           <t>ИЯИ РАН</t>
         </is>
       </c>
-      <c r="G182" s="4" t="inlineStr">
+      <c r="H182" s="4" t="inlineStr">
         <is>
           <t>Расчет характеристик черенковского детектора для контроля пучков протонов, используемых для флэш-терапии</t>
         </is>
@@ -10301,7 +10236,7 @@
           <t>ОИЯИ</t>
         </is>
       </c>
-      <c r="G183" s="4" t="inlineStr">
+      <c r="H183" s="4" t="inlineStr">
         <is>
           <t>Количественная оценка содержания тория и урана в свинце для радиационной защиты методом ИСП-МС</t>
         </is>
@@ -10336,7 +10271,7 @@
           <t>МГУ</t>
         </is>
       </c>
-      <c r="G184" s="4" t="inlineStr">
+      <c r="H184" s="4" t="inlineStr">
         <is>
           <t>Применение деформируемой регистрации изображений в лучевой терапии</t>
         </is>
@@ -10371,7 +10306,7 @@
           <t>СФВУ (Якутия)</t>
         </is>
       </c>
-      <c r="G185" s="4" t="inlineStr">
+      <c r="H185" s="4" t="inlineStr">
         <is>
           <t>Биофизическая модель электрических характеристик эритроцитов при лучевой терапии</t>
         </is>
@@ -10406,7 +10341,7 @@
           <t>ИЯИ РАН</t>
         </is>
       </c>
-      <c r="G186" s="4" t="inlineStr">
+      <c r="H186" s="4" t="inlineStr">
         <is>
           <t>Корректировка и валидация алгоритма оценки прбега протонов в различных матералах на основании КТ-исследований</t>
         </is>
@@ -10441,7 +10376,7 @@
           <t>INR Uzbekistan</t>
         </is>
       </c>
-      <c r="G187" s="4" t="inlineStr">
+      <c r="H187" s="4" t="inlineStr">
         <is>
           <t>Использование гамма-облученного оксида алюминия для изготовления генераторов технеция-99М</t>
         </is>
@@ -10471,7 +10406,7 @@
           <t>Антон Александрович</t>
         </is>
       </c>
-      <c r="G188" s="4" t="inlineStr">
+      <c r="H188" s="4" t="inlineStr">
         <is>
           <t>Фотоядерное получение медицинских изотопов рения на осмиевых и иридиевых мишенях</t>
         </is>
@@ -10506,7 +10441,7 @@
           <t>МГУ</t>
         </is>
       </c>
-      <c r="G189" s="4" t="inlineStr">
+      <c r="H189" s="4" t="inlineStr">
         <is>
           <t>Ядерные реакции на кислороде, углероде, азоте и боре при облучении протонным пучком 160 МэВ</t>
         </is>
@@ -10541,7 +10476,7 @@
           <t>МКНЦ, МГУ</t>
         </is>
       </c>
-      <c r="G190" s="4" t="inlineStr">
+      <c r="H190" s="4" t="inlineStr">
         <is>
           <t>Исследование влияния термопластических масок на поверхностную дозу и дозовое распределение в лучевой терапии</t>
         </is>
@@ -10576,7 +10511,7 @@
           <t>МИФИ, МКНЦ</t>
         </is>
       </c>
-      <c r="G191" s="4" t="inlineStr">
+      <c r="H191" s="4" t="inlineStr">
         <is>
           <t>Биофизическое моделирование распределения температуры при гипертермии: обзор алгоритмов и проектирование расчётного модуля.</t>
         </is>
@@ -10611,7 +10546,7 @@
           <t>ИАЭ Обнинск</t>
         </is>
       </c>
-      <c r="G192" s="4" t="inlineStr">
+      <c r="H192" s="4" t="inlineStr">
         <is>
           <t>Optimization of photoneutron source parameters for boron neutron capture therapy</t>
         </is>
@@ -10646,7 +10581,7 @@
           <t>ТПУ (Томск)</t>
         </is>
       </c>
-      <c r="G193" s="4" t="inlineStr">
+      <c r="H193" s="4" t="inlineStr">
         <is>
           <t>Спектральные измерения пучка быстрых нейтронов циклотрона У-120</t>
         </is>
@@ -10681,7 +10616,7 @@
           <t>РМНЦ им. Цыба</t>
         </is>
       </c>
-      <c r="G194" s="4" t="inlineStr">
+      <c r="H194" s="4" t="inlineStr">
         <is>
           <t>Статус проекта по созданию комплекса нейтронной терапии на базе компактного нейтронного генератора НГ-24МТ</t>
         </is>
@@ -10716,7 +10651,7 @@
           <t>РМНЦ им. Цыба</t>
         </is>
       </c>
-      <c r="G195" s="4" t="inlineStr">
+      <c r="H195" s="4" t="inlineStr">
         <is>
           <t>Особенности вычислительного прогнозирования отклика ионизационных камер для радиотерапевтического применения</t>
         </is>
@@ -10751,7 +10686,7 @@
           <t>МГУ</t>
         </is>
       </c>
-      <c r="G196" s="4" t="inlineStr">
+      <c r="H196" s="4" t="inlineStr">
         <is>
           <t>Моделирование комбинированного воздействия ионизирующего излучения и озона для стерилизации биоматериалов</t>
         </is>
@@ -10786,7 +10721,7 @@
           <t>МГУ</t>
         </is>
       </c>
-      <c r="G197" s="4" t="inlineStr">
+      <c r="H197" s="4" t="inlineStr">
         <is>
           <t>Применение шумоподавляющих фильтров при плёночной дозиметрии радиохирургических планов лечения</t>
         </is>
@@ -10821,7 +10756,7 @@
           <t>МГУ</t>
         </is>
       </c>
-      <c r="G198" s="4" t="inlineStr">
+      <c r="H198" s="4" t="inlineStr">
         <is>
           <t>Методика дозиметрии источника для электронной поверхностной брахитерапии</t>
         </is>
@@ -10856,7 +10791,7 @@
           <t>СФВУ (Якутия)</t>
         </is>
       </c>
-      <c r="G199" s="4" t="inlineStr">
+      <c r="H199" s="4" t="inlineStr">
         <is>
           <t>Накопление золошлаковых отходов и выбросов котельного комплекса и рост онкологической заболеваемости</t>
         </is>
@@ -10878,7 +10813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10915,25 +10850,30 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Название</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Секция</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>№ стенда</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Примечание (RU)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Примечание (EN)</t>
         </is>
@@ -10955,12 +10895,12 @@
           <t>Илья</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Поиск распадов с нарушением принципа Паули и барионного числа с помощью детектора Борексино</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -10982,12 +10922,12 @@
           <t>Alexander</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Estimated B(E2) values for neutron-rich actinide nuclei</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -11009,12 +10949,12 @@
           <t>Alexander</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Binding energy estimates for even-even actinide nuclei</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -11036,12 +10976,12 @@
           <t>Alexander</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Evolution of the neutron shell gap for N&gt;150 with increasing Z from 89 to 100</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -11063,12 +11003,12 @@
           <t>Марат Абжанович</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>О природе низколежащих состояний ядра 7Li</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -11090,12 +11030,12 @@
           <t>Марат Абжанович</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>О связи каналов в потенциальных кластерных моделях</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -11117,12 +11057,12 @@
           <t>Яна Олеговна</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Исследование деформаций предразрывных конфигураций фрагментов при эмиссии третьей легкой частицы</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -11144,12 +11084,12 @@
           <t>Матвей Александрович</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Измерения бета-спектра 99Тс с помощью спектрометра на основе Si(Li)-детекторов</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -11171,12 +11111,12 @@
           <t>Valentine</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Характеристики α-распада неизвестных ядер в области Z ≥ 100</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -11198,12 +11138,12 @@
           <t>Артур Ришатович</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>Влияние тензорных сил на нейтронную шубу в изотопах олова</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -11225,12 +11165,12 @@
           <t>Олег Викторович</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Channeling radiation as a tool for GDR excitation in yttrium</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -11252,12 +11192,12 @@
           <t>Валерий Валерьевич</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Результаты измерения дифференциального сечения образования мгновенных гамма-квантов в реакциях быстрых нейтронов с ядрами титана</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -11279,17 +11219,17 @@
           <t>Александр Викторович</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Результаты моделирования эксперимента по исследованию фотоядерных реакций на источнике комптоновского излучения</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>Соавтор/пометка в исходнике: Гаганов</t>
         </is>
@@ -11311,12 +11251,12 @@
           <t>Егор</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Расчёт сечений образования изомера серебра 108mAg в (d,p) реакциях на ускорителе ЭГП-10</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -11338,12 +11278,12 @@
           <t>Александр Павлович</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Изучение формата ENDF-6 для извлечения ядерных данных по реакциям с нейтронами</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -11365,12 +11305,12 @@
           <t>Александр Александрович</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>Исследование реакции n + 2H → n +n+p при энергии нейтронов 20 МэВ</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -11392,12 +11332,12 @@
           <t>Владимир Т.</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Безнейтринный двойной электронный захват, стимулируемый рентгеновскими лучами</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -11419,12 +11359,12 @@
           <t>Вячеслав Владимирович</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Экспериментальная установка для определения спектра энергии возбуждения ядра 10Be в реакции n + 9Be</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -11446,12 +11386,12 @@
           <t>Сергей</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>Реакции слияния тяжелых ядер для астрофизических задач</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -11473,12 +11413,12 @@
           <t>Абдулмажид Хусейн</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Моделирование и измерение параметров дрейфа электронов в активной мишени</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11500,17 +11440,17 @@
           <t>Александр Евгеньевич</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>Детектор импульсного ионизирующего излучения с субнаносекундным временным разрешением на основе радиационно-наведенного поглощения света в лейкосапфире</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>Соавтор/пометка в исходнике: Залозная</t>
         </is>
@@ -11532,12 +11472,12 @@
           <t>Vyacheslav</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Применение микроконтроллерных и микрокомпьютерных систем в измерительных комплексах на базе стандарта КАМАК</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11559,12 +11499,12 @@
           <t>Shakir</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>Моделирование кросс-толка нейтронов в плотноупакованных сцинтилляционных сборках для экспериментов по множественности мгновенных нейтронов деления</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11586,12 +11526,12 @@
           <t>Егор</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>Диагностика пучков заряженных частиц и определение коэффициентов вторичной электронной эмиссии материалов</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11613,12 +11553,12 @@
           <t>Дарья Андреевна</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Исследование сцинтилляционных детекторов, применяемых в диагностических системах время-пролётной позитронно-эмиссионной томографии</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11640,12 +11580,12 @@
           <t>Анастасия Михайловна</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>Особенности ядерных реакций с получением 99mTc на пучках протонов с энергиями до 100 МэВ</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11667,12 +11607,12 @@
           <t>Дэжуй</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>Стенд для проведения нейтронной активации</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11694,12 +11634,12 @@
           <t>Михаил Вадимович</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>Измерение профиля пучка нейтронного поля центрального нейтронного канала на экспериментальных площадках установки РАДЭКС ИЯИ РАН</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11721,12 +11661,12 @@
           <t>Екатерина Владимировна</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>Применение на ускорительном комплексе У-70</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11748,12 +11688,12 @@
           <t>Анна Станиславовна</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>Перспективы применения сухой ионно-плазменной технологии дезактивации оборудования ЯЭУ из титановых сплавов</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11775,12 +11715,12 @@
           <t>Андрей Александрович</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>Цифровая модель процесса неразрушающего контроля положения пружины в твэле гамма-абсорбционным методом</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11802,12 +11742,12 @@
           <t>Андрей Александрович</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>Анализ влияния локальных неоднородностей топливной таблетки на прохождение гамма-излучения через твэл</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11829,12 +11769,12 @@
           <t>Андрей Александрович</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>Математическое моделирование методов определения флюенса альфа-излучения источника, расположенного на сложной поверхности</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11856,12 +11796,12 @@
           <t>Olga</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>Моделирование кросс-толка нейтронов в плотноупакованных сцинтилляционных сборках для экспериментов по множественности мгновенных нейтронов деления</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11883,12 +11823,12 @@
           <t>Варвара Аркадьевна</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>Фемтосекундная лазерная система для исследования отклика сцинтилляторов γ-излучения</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11910,12 +11850,12 @@
           <t>Юлия Викторовна</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr">
         <is>
           <t>Подготовка малошумящего детектора на микроканальных пластинах для регистрации кумулятивных частиц в экспериментах на фиксированной мишени</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11937,12 +11877,12 @@
           <t>Арсений Игоревич</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="F38" s="4" t="inlineStr">
         <is>
           <t>Study of the correlation function between cells in the HGND at the BM@N experiment</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -11964,12 +11904,12 @@
           <t>Владимир Николаевич</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="F39" s="4" t="inlineStr">
         <is>
           <t>Моделирование подпорогового рождения антипротонов и кумулятивных процессов в столкновениях тяжелых ионов</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -11991,12 +11931,12 @@
           <t>Владимир Николаевич</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr">
         <is>
           <t>Рождение странных частиц в pp- и AA-столкновениях в расширенной модели мультипомеронного обмена</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -12018,12 +11958,12 @@
           <t>Александр Трофимович</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="F41" s="4" t="inlineStr">
         <is>
           <t>Квазиклассическое описание поведения малого числа тел для адронов и темной материи</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -12045,12 +11985,12 @@
           <t>Валентина Николаевна</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="F42" s="4" t="inlineStr">
         <is>
           <t>Поиск бустерной темной материи, ускоренной электронами космических лучей</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -12072,12 +12012,12 @@
           <t>Ангелина-Наталия Валерьевна</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="F43" s="4" t="inlineStr">
         <is>
           <t>Методы раннего обнаружения аномалий в радионуклидных выбросах АЭС на основе статистик многолетнего мониторинга</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12099,12 +12039,12 @@
           <t>Gazimagomed</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>Determination of the distribution coefficients of elements in the diacetyl/hydrochloric acid system for nuclear medicine applications</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12126,12 +12066,12 @@
           <t>Надежда, Анатольевна</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="F45" s="4" t="inlineStr">
         <is>
           <t>Анализ повреждения коллагена в костных биоимплантатах при радиационной стерилизации</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12153,12 +12093,12 @@
           <t>Андрей</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="F46" s="4" t="inlineStr">
         <is>
           <t>Анализ больших массивов радиоэкологических измерений после крупных ядерных аварий: оценка эффективных периодов полувыведения и пространственных закономерностей на открытых данных</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="G46" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12180,12 +12120,12 @@
           <t>Аида</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr">
         <is>
           <t>Математическое моделирование при исследовании материала для коллиматора смешанного гамма-нейтронного пучка циклотрона У-120</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -12207,12 +12147,12 @@
           <t>Sayara</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>Fluctuations and correlations in relativistic nucleus–nucleus collisions</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>4</t>
         </is>

</xml_diff>

<commit_message>
Update .gitignore to include additional Excel report files; revise README.md for clarity on section audience defaults and document swapping instructions; enhance inconsistencies.md with updated audience information and cancellation statuses; improve app.js and common.py for room label expansion and status handling in posters; adjust app.css for poster cancellation styling.
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -21,10 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="DD.MM.YYYY"/>
     <numFmt numFmtId="165" formatCode="HH:MM"/>
     <numFmt numFmtId="166" formatCode="DD.MM.YYYY HH:MM"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -1129,6 +1130,11 @@
           <t>Opening ceremony</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n">
@@ -1165,6 +1171,11 @@
           <t>Ю1</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
@@ -1201,6 +1212,11 @@
           <t>Ю2</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n">
@@ -1263,6 +1279,11 @@
           <t>1</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
@@ -1299,6 +1320,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
@@ -1335,6 +1361,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
@@ -1397,6 +1428,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
@@ -1433,6 +1469,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
@@ -1469,6 +1510,11 @@
           <t>С1</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
@@ -1505,6 +1551,11 @@
           <t>С2</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n">
@@ -1541,6 +1592,11 @@
           <t>С3</t>
         </is>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
@@ -1593,6 +1649,11 @@
           <t>1-7</t>
         </is>
       </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
@@ -1619,6 +1680,11 @@
           <t>1-7</t>
         </is>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>144ц</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
@@ -1645,6 +1711,11 @@
           <t>1-7</t>
         </is>
       </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>117л</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
@@ -1671,6 +1742,11 @@
           <t>1-7</t>
         </is>
       </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>315л</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
@@ -1733,6 +1809,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">
@@ -1769,6 +1850,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n">
@@ -1805,6 +1891,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n">
@@ -1867,6 +1958,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
@@ -1903,6 +1999,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
@@ -1939,6 +2040,11 @@
           <t>11</t>
         </is>
       </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
@@ -1991,6 +2097,11 @@
           <t>8-14</t>
         </is>
       </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
@@ -2017,6 +2128,11 @@
           <t>8-14</t>
         </is>
       </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>144ц</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
@@ -2043,6 +2159,11 @@
           <t>1-7</t>
         </is>
       </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>117л</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
@@ -2069,6 +2190,11 @@
           <t>8-14</t>
         </is>
       </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>315л</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
@@ -2121,6 +2247,11 @@
           <t>15-21</t>
         </is>
       </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>144ц</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n">
@@ -2147,6 +2278,11 @@
           <t>8-14</t>
         </is>
       </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
@@ -2173,6 +2309,11 @@
           <t>8-14</t>
         </is>
       </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>117л</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
@@ -2199,6 +2340,11 @@
           <t>15-21</t>
         </is>
       </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>315л</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
@@ -2261,6 +2407,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
@@ -2297,6 +2448,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n">
@@ -2333,6 +2489,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n">
@@ -2395,6 +2556,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n">
@@ -2431,6 +2597,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
@@ -2467,6 +2638,11 @@
           <t>17</t>
         </is>
       </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
@@ -2519,6 +2695,11 @@
           <t>15-22</t>
         </is>
       </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n">
@@ -2528,7 +2709,7 @@
         <v>0.5833333333333334</v>
       </c>
       <c r="C49" s="7" t="n">
-        <v>0.6770833333333334</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2543,6 +2724,11 @@
       <c r="H49" t="inlineStr">
         <is>
           <t>22-29</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>144ц</t>
         </is>
       </c>
     </row>
@@ -2571,6 +2757,11 @@
           <t>1-9</t>
         </is>
       </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>117л</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="n">
@@ -2580,7 +2771,7 @@
         <v>0.5833333333333334</v>
       </c>
       <c r="C51" s="7" t="n">
-        <v>0.6770833333333334</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2595,6 +2786,11 @@
       <c r="H51" t="inlineStr">
         <is>
           <t>1-8</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>315л</t>
         </is>
       </c>
     </row>
@@ -2695,6 +2891,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n">
@@ -2731,6 +2932,11 @@
           <t>19</t>
         </is>
       </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="n">
@@ -2767,6 +2973,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="n">
@@ -2829,6 +3040,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="n">
@@ -2865,6 +3081,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="n">
@@ -2901,6 +3122,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="6" t="n">
@@ -3015,6 +3241,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="n">
@@ -3051,6 +3282,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="n">
@@ -3087,6 +3323,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="n">
@@ -3149,6 +3390,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="n">
@@ -3185,6 +3431,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="6" t="n">
@@ -3221,6 +3472,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="n">
@@ -3273,16 +3529,21 @@
           <t>23-29</t>
         </is>
       </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="n">
         <v>46290</v>
       </c>
       <c r="B73" s="7" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.6770833333333334</v>
       </c>
       <c r="C73" s="7" t="n">
-        <v>0.65625</v>
+        <v>0.75</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3297,6 +3558,11 @@
       <c r="H73" t="inlineStr">
         <is>
           <t>30-36</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>235ц</t>
         </is>
       </c>
     </row>
@@ -3325,6 +3591,11 @@
           <t>15-21</t>
         </is>
       </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>117л</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="n">
@@ -3351,6 +3622,11 @@
           <t>15-21</t>
         </is>
       </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>144ц</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="6" t="n">
@@ -3403,6 +3679,11 @@
           <t>22-27</t>
         </is>
       </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>117л</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="6" t="n">
@@ -3429,16 +3710,21 @@
           <t>22-28</t>
         </is>
       </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>144ц</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="n">
         <v>46290</v>
       </c>
       <c r="B79" s="7" t="n">
-        <v>0.6770833333333334</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="C79" s="7" t="n">
-        <v>0.75</v>
+        <v>0.6145833333333334</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3453,6 +3739,11 @@
       <c r="H79" t="inlineStr">
         <is>
           <t>22-24</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>315л</t>
         </is>
       </c>
     </row>
@@ -3491,6 +3782,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="n">
@@ -3527,6 +3823,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="n">
@@ -3563,6 +3864,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>235ц</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="6" t="n">
@@ -3613,6 +3919,11 @@
       <c r="F84" t="inlineStr">
         <is>
           <t>Closing ceremony</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>235ц</t>
         </is>
       </c>
     </row>
@@ -4811,6 +5122,11 @@
       <c r="I29" t="n">
         <v>30</v>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>отменён</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>2</t>
@@ -6156,6 +6472,11 @@
           <t>Isotopic dependence of the fission threshold in nuclei with Z=114 and Z=120</t>
         </is>
       </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>отменён</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -6191,6 +6512,11 @@
           <t>Анализ альфа-распадных цепочек элементов 119 и 120 в двухцентровой оболочечной модели: конкуренция незапрещённых и запрещённых переходов</t>
         </is>
       </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>отменён</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6226,6 +6552,11 @@
           <t>Анализ рассеяния дейтронов на ядре 13C в области энергий 13–18 МэВ: структура возбуждённых состояний и нейтронное гало</t>
         </is>
       </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>отменён</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -6506,6 +6837,11 @@
           <t>Status of research on fissioning isomers in the fragments of binary fission of heavy nuclei</t>
         </is>
       </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>отменён</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -8704,6 +9040,11 @@
       <c r="H139" s="4" t="inlineStr">
         <is>
           <t>Эффективность и математические аналоги процедуры ИБП при вычислении интегралов Фейнмана</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>отменён</t>
         </is>
       </c>
     </row>
@@ -10813,7 +11154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10870,10 +11211,15 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Статус</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Примечание (RU)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Примечание (EN)</t>
         </is>
@@ -11231,6 +11577,11 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
+          <t>отменён</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
           <t>Соавтор/пометка в исходнике: Гаганов</t>
         </is>
       </c>
@@ -11396,6 +11747,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>отменён</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -11452,6 +11808,11 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
+          <t>отменён</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
           <t>Соавтор/пометка в исходнике: Залозная</t>
         </is>
       </c>
@@ -11536,6 +11897,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>отменён</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -11563,6 +11929,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>отменён</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -11590,6 +11961,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>отменён</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -12157,8 +12533,18 @@
           <t>4</t>
         </is>
       </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>отменён</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="I2:I248" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"отменён,перенесён"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12169,7 +12555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -12209,6 +12595,21 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="8" t="n">
+        <v>46276.86666666667</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Указаны аудитории. Не приедут (доклады отменены): Варламов, Мардыбан, Безбах А. Н., Данилов, Каманин, Бытьев; постеры Долгополов, Торилов, Дормидонов, Землин, Комарова, Кострыгина, Ibraimova.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Rooms added. Cancelled (will not attend): Varlamov, Mardyban, Bezbakh A. N., Danilov, Kamanin, Bytiev; posters Dolgopolov, Torilov, Dormidonov, Zemlin, Komarova, Kostrygina, Ibraimova.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Modify app.css to enhance font handling for mathematical symbols and improve layout for titles with superscripts and subscripts; update app.js to implement new functions for title formatting and display, ensuring better handling of speaker names and titles; adjust data.js for conference schedule details. Update .gitignore to include additional PDF files;
</commit_message>
<xml_diff>
--- a/data/programme.xlsx
+++ b/data/programme.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="11220" yWindow="3910" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Настройки" sheetId="1" state="visible" r:id="rId1"/>
@@ -15,16 +14,16 @@
     <sheet name="Изменения" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="DD.MM.YYYY"/>
-    <numFmt numFmtId="165" formatCode="HH:MM"/>
-    <numFmt numFmtId="166" formatCode="DD.MM.YYYY HH:MM"/>
+    <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="165" formatCode="hh:mm"/>
+    <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy\ hh:mm"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -35,8 +34,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -48,7 +49,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F2937"/>
+        <fgColor rgb="FF1F2937"/>
       </patternFill>
     </fill>
   </fills>
@@ -64,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -75,12 +76,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -444,11 +442,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="2" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -640,7 +637,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>E-mail или телефон; показывается в подвале</t>
+          <t>E-mail или телефон; показывается в конце</t>
         </is>
       </c>
     </row>
@@ -678,15 +675,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="2" max="3"/>
+    <col width="60" customWidth="1" min="4" max="5"/>
+    <col width="22" customWidth="1" min="6" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
@@ -1006,19 +1000,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K84"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="2" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="5" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="10" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1079,13 +1070,13 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="n">
+      <c r="A2" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B2" s="7" t="n">
+      <c r="B2" s="3" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="C2" s="7" t="n">
+      <c r="C2" s="3" t="n">
         <v>0.375</v>
       </c>
       <c r="D2" t="inlineStr">
@@ -1105,13 +1096,13 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n">
+      <c r="A3" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B3" s="7" t="n">
+      <c r="B3" s="3" t="n">
         <v>0.375</v>
       </c>
-      <c r="C3" s="7" t="n">
+      <c r="C3" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
       <c r="D3" t="inlineStr">
@@ -1136,13 +1127,13 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B4" s="7" t="n">
+      <c r="B4" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="3" t="n">
         <v>0.4166666666666667</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -1177,13 +1168,13 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="3" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="3" t="n">
         <v>0.4375</v>
       </c>
       <c r="D5" t="inlineStr">
@@ -1218,13 +1209,13 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="3" t="n">
         <v>0.4375</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="3" t="n">
         <v>0.4583333333333333</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -1244,13 +1235,13 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="3" t="n">
         <v>0.4583333333333333</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -1285,13 +1276,13 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="3" t="n">
         <v>0.5</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -1326,13 +1317,13 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="3" t="n">
         <v>0.5208333333333334</v>
       </c>
       <c r="D9" t="inlineStr">
@@ -1367,13 +1358,13 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="3" t="n">
         <v>0.5208333333333334</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
       <c r="D10" t="inlineStr">
@@ -1393,13 +1384,13 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="3" t="n">
         <v>0.6041666666666666</v>
       </c>
       <c r="D11" t="inlineStr">
@@ -1434,13 +1425,13 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="3" t="n">
         <v>0.6041666666666666</v>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="3" t="n">
         <v>0.625</v>
       </c>
       <c r="D12" t="inlineStr">
@@ -1475,13 +1466,13 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="3" t="n">
         <v>0.625</v>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="3" t="n">
         <v>0.6354166666666666</v>
       </c>
       <c r="D13" t="inlineStr">
@@ -1516,13 +1507,13 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="3" t="n">
         <v>0.6354166666666666</v>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="3" t="n">
         <v>0.6458333333333334</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -1557,13 +1548,13 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="3" t="n">
         <v>0.6458333333333334</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="3" t="n">
         <v>0.65625</v>
       </c>
       <c r="D15" t="inlineStr">
@@ -1598,13 +1589,13 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B16" s="7" t="n">
+      <c r="B16" s="3" t="n">
         <v>0.65625</v>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
       <c r="D16" t="inlineStr">
@@ -1624,13 +1615,13 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="n">
+      <c r="A17" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B17" s="7" t="n">
+      <c r="B17" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C17" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="D17" t="inlineStr">
@@ -1655,13 +1646,13 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="n">
+      <c r="A18" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B18" s="7" t="n">
+      <c r="B18" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="C18" s="7" t="n">
+      <c r="C18" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="D18" t="inlineStr">
@@ -1686,13 +1677,13 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="n">
+      <c r="A19" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B19" s="7" t="n">
+      <c r="B19" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="C19" s="7" t="n">
+      <c r="C19" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="D19" t="inlineStr">
@@ -1717,13 +1708,13 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="n">
+      <c r="A20" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B20" s="7" t="n">
+      <c r="B20" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="C20" s="7" t="n">
+      <c r="C20" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="D20" t="inlineStr">
@@ -1748,13 +1739,13 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="n">
+      <c r="A21" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="B21" s="7" t="n">
+      <c r="B21" s="3" t="n">
         <v>0.7708333333333334</v>
       </c>
-      <c r="C21" s="7" t="n">
+      <c r="C21" s="3" t="n">
         <v>0.8541666666666666</v>
       </c>
       <c r="D21" t="inlineStr">
@@ -1774,13 +1765,13 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="n">
+      <c r="A22" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B22" s="7" t="n">
+      <c r="B22" s="3" t="n">
         <v>0.375</v>
       </c>
-      <c r="C22" s="7" t="n">
+      <c r="C22" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
       <c r="D22" t="inlineStr">
@@ -1815,13 +1806,13 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="n">
+      <c r="A23" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B23" s="7" t="n">
+      <c r="B23" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
-      <c r="C23" s="7" t="n">
+      <c r="C23" s="3" t="n">
         <v>0.4166666666666667</v>
       </c>
       <c r="D23" t="inlineStr">
@@ -1856,13 +1847,13 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="n">
+      <c r="A24" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B24" s="7" t="n">
+      <c r="B24" s="3" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="C24" s="7" t="n">
+      <c r="C24" s="3" t="n">
         <v>0.4375</v>
       </c>
       <c r="D24" t="inlineStr">
@@ -1897,13 +1888,13 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="n">
+      <c r="A25" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B25" s="7" t="n">
+      <c r="B25" s="3" t="n">
         <v>0.4375</v>
       </c>
-      <c r="C25" s="7" t="n">
+      <c r="C25" s="3" t="n">
         <v>0.4583333333333333</v>
       </c>
       <c r="D25" t="inlineStr">
@@ -1923,13 +1914,13 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="n">
+      <c r="A26" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B26" s="7" t="n">
+      <c r="B26" s="3" t="n">
         <v>0.4583333333333333</v>
       </c>
-      <c r="C26" s="7" t="n">
+      <c r="C26" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
       <c r="D26" t="inlineStr">
@@ -1964,13 +1955,13 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="n">
+      <c r="A27" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B27" s="7" t="n">
+      <c r="B27" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C27" s="7" t="n">
+      <c r="C27" s="3" t="n">
         <v>0.5</v>
       </c>
       <c r="D27" t="inlineStr">
@@ -2005,13 +1996,13 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="n">
+      <c r="A28" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B28" s="7" t="n">
+      <c r="B28" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="C28" s="7" t="n">
+      <c r="C28" s="3" t="n">
         <v>0.5208333333333334</v>
       </c>
       <c r="D28" t="inlineStr">
@@ -2046,13 +2037,13 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="n">
+      <c r="A29" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B29" s="7" t="n">
+      <c r="B29" s="3" t="n">
         <v>0.5208333333333334</v>
       </c>
-      <c r="C29" s="7" t="n">
+      <c r="C29" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
       <c r="D29" t="inlineStr">
@@ -2072,13 +2063,13 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="n">
+      <c r="A30" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B30" s="7" t="n">
+      <c r="B30" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C30" s="7" t="n">
+      <c r="C30" s="3" t="n">
         <v>0.65625</v>
       </c>
       <c r="D30" t="inlineStr">
@@ -2103,13 +2094,13 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="n">
+      <c r="A31" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B31" s="7" t="n">
+      <c r="B31" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C31" s="7" t="n">
+      <c r="C31" s="3" t="n">
         <v>0.65625</v>
       </c>
       <c r="D31" t="inlineStr">
@@ -2134,13 +2125,13 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="n">
+      <c r="A32" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B32" s="7" t="n">
+      <c r="B32" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C32" s="7" t="n">
+      <c r="C32" s="3" t="n">
         <v>0.65625</v>
       </c>
       <c r="D32" t="inlineStr">
@@ -2165,13 +2156,13 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="n">
+      <c r="A33" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B33" s="7" t="n">
+      <c r="B33" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C33" s="7" t="n">
+      <c r="C33" s="3" t="n">
         <v>0.65625</v>
       </c>
       <c r="D33" t="inlineStr">
@@ -2196,13 +2187,13 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="n">
+      <c r="A34" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B34" s="7" t="n">
+      <c r="B34" s="3" t="n">
         <v>0.65625</v>
       </c>
-      <c r="C34" s="7" t="n">
+      <c r="C34" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
       <c r="D34" t="inlineStr">
@@ -2222,13 +2213,13 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="n">
+      <c r="A35" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B35" s="7" t="n">
+      <c r="B35" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="C35" s="7" t="n">
+      <c r="C35" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="D35" t="inlineStr">
@@ -2253,13 +2244,13 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="n">
+      <c r="A36" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B36" s="7" t="n">
+      <c r="B36" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="C36" s="7" t="n">
+      <c r="C36" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="D36" t="inlineStr">
@@ -2284,13 +2275,13 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="n">
+      <c r="A37" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B37" s="7" t="n">
+      <c r="B37" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="C37" s="7" t="n">
+      <c r="C37" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="D37" t="inlineStr">
@@ -2315,13 +2306,13 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="n">
+      <c r="A38" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B38" s="7" t="n">
+      <c r="B38" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="C38" s="7" t="n">
+      <c r="C38" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="D38" t="inlineStr">
@@ -2346,13 +2337,13 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="n">
+      <c r="A39" s="2" t="n">
         <v>46287</v>
       </c>
-      <c r="B39" s="7" t="n">
+      <c r="B39" s="3" t="n">
         <v>0.7708333333333334</v>
       </c>
-      <c r="C39" s="7" t="n">
+      <c r="C39" s="3" t="n">
         <v>0.8125</v>
       </c>
       <c r="D39" t="inlineStr">
@@ -2372,13 +2363,13 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="n">
+      <c r="A40" s="2" t="n">
         <v>46288</v>
       </c>
-      <c r="B40" s="7" t="n">
+      <c r="B40" s="3" t="n">
         <v>0.375</v>
       </c>
-      <c r="C40" s="7" t="n">
+      <c r="C40" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
       <c r="D40" t="inlineStr">
@@ -2413,13 +2404,13 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="n">
+      <c r="A41" s="2" t="n">
         <v>46288</v>
       </c>
-      <c r="B41" s="7" t="n">
+      <c r="B41" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
-      <c r="C41" s="7" t="n">
+      <c r="C41" s="3" t="n">
         <v>0.4166666666666667</v>
       </c>
       <c r="D41" t="inlineStr">
@@ -2454,13 +2445,13 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="n">
+      <c r="A42" s="2" t="n">
         <v>46288</v>
       </c>
-      <c r="B42" s="7" t="n">
+      <c r="B42" s="3" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="C42" s="7" t="n">
+      <c r="C42" s="3" t="n">
         <v>0.4375</v>
       </c>
       <c r="D42" t="inlineStr">
@@ -2495,13 +2486,13 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="n">
+      <c r="A43" s="2" t="n">
         <v>46288</v>
       </c>
-      <c r="B43" s="7" t="n">
+      <c r="B43" s="3" t="n">
         <v>0.4375</v>
       </c>
-      <c r="C43" s="7" t="n">
+      <c r="C43" s="3" t="n">
         <v>0.4583333333333333</v>
       </c>
       <c r="D43" t="inlineStr">
@@ -2521,13 +2512,13 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="n">
+      <c r="A44" s="2" t="n">
         <v>46288</v>
       </c>
-      <c r="B44" s="7" t="n">
+      <c r="B44" s="3" t="n">
         <v>0.4583333333333333</v>
       </c>
-      <c r="C44" s="7" t="n">
+      <c r="C44" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
       <c r="D44" t="inlineStr">
@@ -2562,13 +2553,13 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="n">
+      <c r="A45" s="2" t="n">
         <v>46288</v>
       </c>
-      <c r="B45" s="7" t="n">
+      <c r="B45" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C45" s="7" t="n">
+      <c r="C45" s="3" t="n">
         <v>0.5</v>
       </c>
       <c r="D45" t="inlineStr">
@@ -2603,13 +2594,13 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="n">
+      <c r="A46" s="2" t="n">
         <v>46288</v>
       </c>
-      <c r="B46" s="7" t="n">
+      <c r="B46" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="C46" s="7" t="n">
+      <c r="C46" s="3" t="n">
         <v>0.5208333333333334</v>
       </c>
       <c r="D46" t="inlineStr">
@@ -2644,13 +2635,13 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="n">
+      <c r="A47" s="2" t="n">
         <v>46288</v>
       </c>
-      <c r="B47" s="7" t="n">
+      <c r="B47" s="3" t="n">
         <v>0.5208333333333334</v>
       </c>
-      <c r="C47" s="7" t="n">
+      <c r="C47" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
       <c r="D47" t="inlineStr">
@@ -2670,13 +2661,13 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="n">
+      <c r="A48" s="2" t="n">
         <v>46288</v>
       </c>
-      <c r="B48" s="7" t="n">
+      <c r="B48" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C48" s="7" t="n">
+      <c r="C48" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
       <c r="D48" t="inlineStr">
@@ -2701,13 +2692,13 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="n">
+      <c r="A49" s="2" t="n">
         <v>46288</v>
       </c>
-      <c r="B49" s="7" t="n">
+      <c r="B49" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C49" s="7" t="n">
+      <c r="C49" s="3" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="D49" t="inlineStr">
@@ -2732,13 +2723,13 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="n">
+      <c r="A50" s="2" t="n">
         <v>46288</v>
       </c>
-      <c r="B50" s="7" t="n">
+      <c r="B50" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C50" s="7" t="n">
+      <c r="C50" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
       <c r="D50" t="inlineStr">
@@ -2763,13 +2754,13 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="n">
+      <c r="A51" s="2" t="n">
         <v>46288</v>
       </c>
-      <c r="B51" s="7" t="n">
+      <c r="B51" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C51" s="7" t="n">
+      <c r="C51" s="3" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="D51" t="inlineStr">
@@ -2794,13 +2785,13 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="n">
+      <c r="A52" s="2" t="n">
         <v>46288</v>
       </c>
-      <c r="B52" s="7" t="n">
+      <c r="B52" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="C52" s="7" t="n">
+      <c r="C52" s="3" t="n">
         <v>0.6979166666666666</v>
       </c>
       <c r="D52" t="inlineStr">
@@ -2820,13 +2811,13 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="n">
+      <c r="A53" s="2" t="n">
         <v>46288</v>
       </c>
-      <c r="B53" s="7" t="n">
+      <c r="B53" s="3" t="n">
         <v>0.6979166666666666</v>
       </c>
-      <c r="C53" s="7" t="n">
+      <c r="C53" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="D53" t="inlineStr">
@@ -2856,13 +2847,13 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="n">
+      <c r="A54" s="2" t="n">
         <v>46289</v>
       </c>
-      <c r="B54" s="7" t="n">
+      <c r="B54" s="3" t="n">
         <v>0.375</v>
       </c>
-      <c r="C54" s="7" t="n">
+      <c r="C54" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
       <c r="D54" t="inlineStr">
@@ -2897,13 +2888,13 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="n">
+      <c r="A55" s="2" t="n">
         <v>46289</v>
       </c>
-      <c r="B55" s="7" t="n">
+      <c r="B55" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
-      <c r="C55" s="7" t="n">
+      <c r="C55" s="3" t="n">
         <v>0.4166666666666667</v>
       </c>
       <c r="D55" t="inlineStr">
@@ -2938,13 +2929,13 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="n">
+      <c r="A56" s="2" t="n">
         <v>46289</v>
       </c>
-      <c r="B56" s="7" t="n">
+      <c r="B56" s="3" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="C56" s="7" t="n">
+      <c r="C56" s="3" t="n">
         <v>0.4375</v>
       </c>
       <c r="D56" t="inlineStr">
@@ -2979,13 +2970,13 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="n">
+      <c r="A57" s="2" t="n">
         <v>46289</v>
       </c>
-      <c r="B57" s="7" t="n">
+      <c r="B57" s="3" t="n">
         <v>0.4375</v>
       </c>
-      <c r="C57" s="7" t="n">
+      <c r="C57" s="3" t="n">
         <v>0.4583333333333333</v>
       </c>
       <c r="D57" t="inlineStr">
@@ -3005,13 +2996,13 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="n">
+      <c r="A58" s="2" t="n">
         <v>46289</v>
       </c>
-      <c r="B58" s="7" t="n">
+      <c r="B58" s="3" t="n">
         <v>0.4583333333333333</v>
       </c>
-      <c r="C58" s="7" t="n">
+      <c r="C58" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
       <c r="D58" t="inlineStr">
@@ -3046,13 +3037,13 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="n">
+      <c r="A59" s="2" t="n">
         <v>46289</v>
       </c>
-      <c r="B59" s="7" t="n">
+      <c r="B59" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C59" s="7" t="n">
+      <c r="C59" s="3" t="n">
         <v>0.5</v>
       </c>
       <c r="D59" t="inlineStr">
@@ -3087,13 +3078,13 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="n">
+      <c r="A60" s="2" t="n">
         <v>46289</v>
       </c>
-      <c r="B60" s="7" t="n">
+      <c r="B60" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="C60" s="7" t="n">
+      <c r="C60" s="3" t="n">
         <v>0.5208333333333334</v>
       </c>
       <c r="D60" t="inlineStr">
@@ -3128,13 +3119,13 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="6" t="n">
+      <c r="A61" s="2" t="n">
         <v>46289</v>
       </c>
-      <c r="B61" s="7" t="n">
+      <c r="B61" s="3" t="n">
         <v>0.5208333333333334</v>
       </c>
-      <c r="C61" s="7" t="n">
+      <c r="C61" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
       <c r="D61" t="inlineStr">
@@ -3154,13 +3145,13 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="n">
+      <c r="A62" s="2" t="n">
         <v>46289</v>
       </c>
-      <c r="B62" s="7" t="n">
+      <c r="B62" s="3" t="n">
         <v>0.625</v>
       </c>
-      <c r="C62" s="7" t="n">
+      <c r="C62" s="3" t="n">
         <v>0.7291666666666666</v>
       </c>
       <c r="D62" t="inlineStr">
@@ -3180,13 +3171,13 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="6" t="n">
+      <c r="A63" s="2" t="n">
         <v>46289</v>
       </c>
-      <c r="B63" s="7" t="n">
+      <c r="B63" s="3" t="n">
         <v>0.7916666666666666</v>
       </c>
-      <c r="C63" s="7" t="n">
+      <c r="C63" s="3" t="n">
         <v>0.8958333333333334</v>
       </c>
       <c r="D63" t="inlineStr">
@@ -3206,13 +3197,13 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="n">
+      <c r="A64" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B64" s="7" t="n">
+      <c r="B64" s="3" t="n">
         <v>0.375</v>
       </c>
-      <c r="C64" s="7" t="n">
+      <c r="C64" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
       <c r="D64" t="inlineStr">
@@ -3247,13 +3238,13 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="n">
+      <c r="A65" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B65" s="7" t="n">
+      <c r="B65" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
-      <c r="C65" s="7" t="n">
+      <c r="C65" s="3" t="n">
         <v>0.4166666666666667</v>
       </c>
       <c r="D65" t="inlineStr">
@@ -3288,13 +3279,13 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="n">
+      <c r="A66" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B66" s="7" t="n">
+      <c r="B66" s="3" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="C66" s="7" t="n">
+      <c r="C66" s="3" t="n">
         <v>0.4375</v>
       </c>
       <c r="D66" t="inlineStr">
@@ -3329,13 +3320,13 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="6" t="n">
+      <c r="A67" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B67" s="7" t="n">
+      <c r="B67" s="3" t="n">
         <v>0.4375</v>
       </c>
-      <c r="C67" s="7" t="n">
+      <c r="C67" s="3" t="n">
         <v>0.4583333333333333</v>
       </c>
       <c r="D67" t="inlineStr">
@@ -3355,13 +3346,13 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="6" t="n">
+      <c r="A68" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B68" s="7" t="n">
+      <c r="B68" s="3" t="n">
         <v>0.4583333333333333</v>
       </c>
-      <c r="C68" s="7" t="n">
+      <c r="C68" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
       <c r="D68" t="inlineStr">
@@ -3396,13 +3387,13 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="6" t="n">
+      <c r="A69" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B69" s="7" t="n">
+      <c r="B69" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C69" s="7" t="n">
+      <c r="C69" s="3" t="n">
         <v>0.5</v>
       </c>
       <c r="D69" t="inlineStr">
@@ -3437,13 +3428,13 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="6" t="n">
+      <c r="A70" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B70" s="7" t="n">
+      <c r="B70" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="C70" s="7" t="n">
+      <c r="C70" s="3" t="n">
         <v>0.5208333333333334</v>
       </c>
       <c r="D70" t="inlineStr">
@@ -3478,13 +3469,13 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="6" t="n">
+      <c r="A71" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B71" s="7" t="n">
+      <c r="B71" s="3" t="n">
         <v>0.5208333333333334</v>
       </c>
-      <c r="C71" s="7" t="n">
+      <c r="C71" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
       <c r="D71" t="inlineStr">
@@ -3504,13 +3495,13 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="6" t="n">
+      <c r="A72" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B72" s="7" t="n">
+      <c r="B72" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C72" s="7" t="n">
+      <c r="C72" s="3" t="n">
         <v>0.65625</v>
       </c>
       <c r="D72" t="inlineStr">
@@ -3535,13 +3526,13 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="6" t="n">
+      <c r="A73" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B73" s="7" t="n">
+      <c r="B73" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="C73" s="7" t="n">
+      <c r="C73" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="D73" t="inlineStr">
@@ -3566,13 +3557,13 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="6" t="n">
+      <c r="A74" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B74" s="7" t="n">
+      <c r="B74" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C74" s="7" t="n">
+      <c r="C74" s="3" t="n">
         <v>0.65625</v>
       </c>
       <c r="D74" t="inlineStr">
@@ -3597,13 +3588,13 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="6" t="n">
+      <c r="A75" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B75" s="7" t="n">
+      <c r="B75" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C75" s="7" t="n">
+      <c r="C75" s="3" t="n">
         <v>0.65625</v>
       </c>
       <c r="D75" t="inlineStr">
@@ -3628,13 +3619,13 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="6" t="n">
+      <c r="A76" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B76" s="7" t="n">
+      <c r="B76" s="3" t="n">
         <v>0.65625</v>
       </c>
-      <c r="C76" s="7" t="n">
+      <c r="C76" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
       <c r="D76" t="inlineStr">
@@ -3654,13 +3645,13 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="6" t="n">
+      <c r="A77" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B77" s="7" t="n">
+      <c r="B77" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="C77" s="7" t="n">
+      <c r="C77" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="D77" t="inlineStr">
@@ -3685,13 +3676,13 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="6" t="n">
+      <c r="A78" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B78" s="7" t="n">
+      <c r="B78" s="3" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="C78" s="7" t="n">
+      <c r="C78" s="3" t="n">
         <v>0.75</v>
       </c>
       <c r="D78" t="inlineStr">
@@ -3716,13 +3707,13 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="6" t="n">
+      <c r="A79" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="B79" s="7" t="n">
+      <c r="B79" s="3" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C79" s="7" t="n">
+      <c r="C79" s="3" t="n">
         <v>0.6145833333333334</v>
       </c>
       <c r="D79" t="inlineStr">
@@ -3747,13 +3738,13 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="6" t="n">
+      <c r="A80" s="2" t="n">
         <v>46291</v>
       </c>
-      <c r="B80" s="7" t="n">
+      <c r="B80" s="3" t="n">
         <v>0.375</v>
       </c>
-      <c r="C80" s="7" t="n">
+      <c r="C80" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
       <c r="D80" t="inlineStr">
@@ -3788,13 +3779,13 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="6" t="n">
+      <c r="A81" s="2" t="n">
         <v>46291</v>
       </c>
-      <c r="B81" s="7" t="n">
+      <c r="B81" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
-      <c r="C81" s="7" t="n">
+      <c r="C81" s="3" t="n">
         <v>0.4166666666666667</v>
       </c>
       <c r="D81" t="inlineStr">
@@ -3829,13 +3820,13 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="6" t="n">
+      <c r="A82" s="2" t="n">
         <v>46291</v>
       </c>
-      <c r="B82" s="7" t="n">
+      <c r="B82" s="3" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="C82" s="7" t="n">
+      <c r="C82" s="3" t="n">
         <v>0.4375</v>
       </c>
       <c r="D82" t="inlineStr">
@@ -3870,13 +3861,13 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="6" t="n">
+      <c r="A83" s="2" t="n">
         <v>46291</v>
       </c>
-      <c r="B83" s="7" t="n">
+      <c r="B83" s="3" t="n">
         <v>0.4375</v>
       </c>
-      <c r="C83" s="7" t="n">
+      <c r="C83" s="3" t="n">
         <v>0.4583333333333333</v>
       </c>
       <c r="D83" t="inlineStr">
@@ -3896,13 +3887,13 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="6" t="n">
+      <c r="A84" s="2" t="n">
         <v>46291</v>
       </c>
-      <c r="B84" s="7" t="n">
+      <c r="B84" s="3" t="n">
         <v>0.4583333333333333</v>
       </c>
-      <c r="C84" s="7" t="n">
+      <c r="C84" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
       <c r="D84" t="inlineStr">
@@ -3943,7 +3934,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O198"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
@@ -3956,8 +3947,7 @@
     <col width="8" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="12" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4037,7 +4027,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="43.5" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
           <t>P-J1</t>
@@ -4082,7 +4072,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="29" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>P-J2</t>
@@ -4127,7 +4117,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="116" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
           <t>P-01</t>
@@ -4177,7 +4167,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="130.5" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>P-02</t>
@@ -4222,7 +4212,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="87" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
           <t>P-03</t>
@@ -4272,7 +4262,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="290" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>P-04</t>
@@ -4322,7 +4312,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="232" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
           <t>P-05</t>
@@ -4372,7 +4362,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="409.5" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>P-S1</t>
@@ -4417,7 +4407,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="174" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
           <t>P-S2</t>
@@ -4462,7 +4452,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="72.5" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
           <t>P-S3</t>
@@ -4502,7 +4492,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="261" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
           <t>P-06</t>
@@ -4552,7 +4542,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="145" customHeight="1">
       <c r="A13" t="inlineStr">
         <is>
           <t>P-07</t>
@@ -4602,7 +4592,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="145" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
           <t>P-08</t>
@@ -4652,7 +4642,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="203" customHeight="1">
       <c r="A15" t="inlineStr">
         <is>
           <t>P-09</t>
@@ -4702,7 +4692,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="203" customHeight="1">
       <c r="A16" t="inlineStr">
         <is>
           <t>P-10</t>
@@ -4752,7 +4742,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="174" customHeight="1">
       <c r="A17" t="inlineStr">
         <is>
           <t>P-11</t>
@@ -4802,7 +4792,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="87" customHeight="1">
       <c r="A18" t="inlineStr">
         <is>
           <t>P-12</t>
@@ -4852,7 +4842,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="232" customHeight="1">
       <c r="A19" t="inlineStr">
         <is>
           <t>P-13</t>
@@ -4902,7 +4892,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="217.5" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
           <t>P-14</t>
@@ -4952,7 +4942,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="203" customHeight="1">
       <c r="A21" t="inlineStr">
         <is>
           <t>P-15</t>
@@ -5002,7 +4992,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="145" customHeight="1">
       <c r="A22" t="inlineStr">
         <is>
           <t>P-16</t>
@@ -5052,7 +5042,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="101.5" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
           <t>P-17</t>
@@ -5102,7 +5092,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="87" customHeight="1">
       <c r="A24" t="inlineStr">
         <is>
           <t>P-18</t>
@@ -5152,7 +5142,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="174" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
           <t>P-19</t>
@@ -5202,7 +5192,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="261" customHeight="1">
       <c r="A26" t="inlineStr">
         <is>
           <t>P-20</t>
@@ -5252,7 +5242,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="145" customHeight="1">
       <c r="A27" t="inlineStr">
         <is>
           <t>P-21</t>
@@ -5302,7 +5292,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="290" customHeight="1">
       <c r="A28" t="inlineStr">
         <is>
           <t>P-22</t>
@@ -5352,7 +5342,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="145" customHeight="1">
       <c r="A29" t="inlineStr">
         <is>
           <t>P-23</t>
@@ -5407,7 +5397,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="72.5" customHeight="1">
       <c r="A30" t="inlineStr">
         <is>
           <t>P-24</t>
@@ -5452,7 +5442,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="348" customHeight="1">
       <c r="A31" t="inlineStr">
         <is>
           <t>P-25</t>
@@ -5502,7 +5492,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="275.5" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
           <t>P-26</t>
@@ -5552,7 +5542,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="174" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
           <t>P-27</t>
@@ -5602,7 +5592,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="116" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
           <t>P-28</t>
@@ -5652,7 +5642,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="130.5" customHeight="1">
       <c r="A35" t="inlineStr">
         <is>
           <t>P-29</t>
@@ -5702,7 +5692,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="87" customHeight="1">
       <c r="A36" t="inlineStr">
         <is>
           <t>P-30</t>
@@ -5747,7 +5737,7 @@
         </is>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="217.5" customHeight="1">
       <c r="A37" t="inlineStr">
         <is>
           <t>P-31</t>
@@ -5797,7 +5787,7 @@
         </is>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="304.5" customHeight="1">
       <c r="A38" t="inlineStr">
         <is>
           <t>P-32</t>
@@ -5847,7 +5837,7 @@
         </is>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="217.5" customHeight="1">
       <c r="A39" t="inlineStr">
         <is>
           <t>S1-01</t>
@@ -5892,7 +5882,7 @@
         </is>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="217.5" customHeight="1">
       <c r="A40" t="inlineStr">
         <is>
           <t>S1-02</t>
@@ -5937,7 +5927,7 @@
         </is>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="174" customHeight="1">
       <c r="A41" t="inlineStr">
         <is>
           <t>S1-03</t>
@@ -5977,7 +5967,7 @@
         </is>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="116" customHeight="1">
       <c r="A42" t="inlineStr">
         <is>
           <t>S1-04</t>
@@ -6022,7 +6012,7 @@
         </is>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="409.5" customHeight="1">
       <c r="A43" t="inlineStr">
         <is>
           <t>S1-05</t>
@@ -6058,11 +6048,11 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Экспериментальная и расчетная зависимости коэффициента внутренней конверсии электрон-позитронной пары от угла их разлета при испускании ее из высоко возбужденного ядра 8Ве*</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
+          <t>Экспериментальная и расчетная зависимости коэффициента внутренней конверсии электрон-позитронной пары от угла их разлета при испускании ее из высоко возбужденного ядра ⁸Ве*</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="348" customHeight="1">
       <c r="A44" t="inlineStr">
         <is>
           <t>S1-06</t>
@@ -6102,7 +6092,7 @@
         </is>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="159.5" customHeight="1">
       <c r="A45" t="inlineStr">
         <is>
           <t>S1-07</t>
@@ -6143,11 +6133,11 @@
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Neural Network Extrapolation of NCSM Results for the 17C Nuclear Spectrum</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
+          <t>Neural Network Extrapolation of NCSM Results for the ¹⁷C Nuclear Spectrum</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="174" customHeight="1">
       <c r="A46" t="inlineStr">
         <is>
           <t>S1-08</t>
@@ -6192,7 +6182,7 @@
         </is>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="246.5" customHeight="1">
       <c r="A47" t="inlineStr">
         <is>
           <t>S1-09</t>
@@ -6237,7 +6227,7 @@
         </is>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="377" customHeight="1">
       <c r="A48" t="inlineStr">
         <is>
           <t>S1-10</t>
@@ -6278,11 +6268,11 @@
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>GEANT4-моделирование экспериментальной установки «Монумент». Выбор оптимальной толщины мишени 136BaCO3 в исследовании обычного мюонного захвата</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
+          <t>GEANT4-моделирование экспериментальной установки «Монумент». Выбор оптимальной толщины мишени ¹³⁶BaCO3 в исследовании обычного мюонного захвата</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="159.5" customHeight="1">
       <c r="A49" t="inlineStr">
         <is>
           <t>S1-11</t>
@@ -6327,7 +6317,7 @@
         </is>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="159.5" customHeight="1">
       <c r="A50" t="inlineStr">
         <is>
           <t>S1-12</t>
@@ -6372,7 +6362,7 @@
         </is>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="72.5" customHeight="1">
       <c r="A51" t="inlineStr">
         <is>
           <t>S1-13</t>
@@ -6408,11 +6398,11 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>Мюонный захват на ядре 136Ba</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
+          <t>Мюонный захват на ядре ¹³⁶Ba</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="304.5" customHeight="1">
       <c r="A52" t="inlineStr">
         <is>
           <t>S1-14</t>
@@ -6457,7 +6447,7 @@
         </is>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="116" customHeight="1">
       <c r="A53" t="inlineStr">
         <is>
           <t>S1-15</t>
@@ -6502,7 +6492,7 @@
         </is>
       </c>
     </row>
-    <row r="54">
+    <row r="54" ht="87" customHeight="1">
       <c r="A54" t="inlineStr">
         <is>
           <t>S1-16</t>
@@ -6542,7 +6532,7 @@
         </is>
       </c>
     </row>
-    <row r="55">
+    <row r="55" ht="203" customHeight="1">
       <c r="A55" t="inlineStr">
         <is>
           <t>S1-17</t>
@@ -6587,7 +6577,7 @@
         </is>
       </c>
     </row>
-    <row r="56">
+    <row r="56" ht="203" customHeight="1">
       <c r="A56" t="inlineStr">
         <is>
           <t>S1-18</t>
@@ -6632,7 +6622,7 @@
         </is>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="174" customHeight="1">
       <c r="A57" t="inlineStr">
         <is>
           <t>S1-19</t>
@@ -6668,11 +6658,11 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>Коэффициенты δ(Е2/М1) для переходов из вибрационных состояний в 182,184W</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
+          <t>Коэффициенты δ(Е2/М1) для переходов из вибрационных состояний в ¹⁸²⸴ ¹⁸⁴W</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="246.5" customHeight="1">
       <c r="A58" t="inlineStr">
         <is>
           <t>S1-20</t>
@@ -6712,7 +6702,7 @@
         </is>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="87" customHeight="1">
       <c r="A59" t="inlineStr">
         <is>
           <t>S1-21</t>
@@ -6753,11 +6743,11 @@
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>Gamma de-excitation of 90mZr isomer</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
+          <t>Gamma de-excitation of ⁹⁰mZr isomer</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="145" customHeight="1">
       <c r="A60" t="inlineStr">
         <is>
           <t>S1-22</t>
@@ -6802,7 +6792,7 @@
         </is>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="174" customHeight="1">
       <c r="A61" t="inlineStr">
         <is>
           <t>S1-23</t>
@@ -6843,11 +6833,11 @@
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>Exploring the superheavy nuclei using 50Ti and 54Cr beams as the projectile</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
+          <t>Exploring the superheavy nuclei using ⁵⁰Ti and ⁵⁴Cr beams as the projectile</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="261" customHeight="1">
       <c r="A62" t="inlineStr">
         <is>
           <t>S1-24</t>
@@ -6892,7 +6882,7 @@
         </is>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="101.5" customHeight="1">
       <c r="A63" t="inlineStr">
         <is>
           <t>S1-25</t>
@@ -6932,7 +6922,7 @@
         </is>
       </c>
     </row>
-    <row r="64">
+    <row r="64" ht="261" customHeight="1">
       <c r="A64" t="inlineStr">
         <is>
           <t>S1-26</t>
@@ -6972,7 +6962,7 @@
         </is>
       </c>
     </row>
-    <row r="65">
+    <row r="65" ht="116" customHeight="1">
       <c r="A65" t="inlineStr">
         <is>
           <t>S1-27</t>
@@ -7013,11 +7003,11 @@
       </c>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>Transition densities of spin-dipole excitations in 208Pb</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
+          <t>Transition densities of spin-dipole excitations in ²⁰⁸Pb</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="174" customHeight="1">
       <c r="A66" t="inlineStr">
         <is>
           <t>S1-28</t>
@@ -7067,7 +7057,7 @@
         </is>
       </c>
     </row>
-    <row r="67">
+    <row r="67" ht="319" customHeight="1">
       <c r="A67" t="inlineStr">
         <is>
           <t>S1-29</t>
@@ -7117,7 +7107,7 @@
         </is>
       </c>
     </row>
-    <row r="68">
+    <row r="68" ht="290" customHeight="1">
       <c r="A68" t="inlineStr">
         <is>
           <t>S2-01</t>
@@ -7158,7 +7148,7 @@
       </c>
       <c r="I68" s="4" t="inlineStr">
         <is>
-          <t>Анализ рассеяния дейтронов на ядре 13C в области энергий 13–18 МэВ: структура возбуждённых состояний и нейтронное гало</t>
+          <t>Анализ рассеяния дейтронов на ядре ¹³C в области энергий 13–18 МэВ: структура возбуждённых состояний и нейтронное гало</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
@@ -7167,7 +7157,7 @@
         </is>
       </c>
     </row>
-    <row r="69">
+    <row r="69" ht="362.5" customHeight="1">
       <c r="A69" t="inlineStr">
         <is>
           <t>S2-02</t>
@@ -7208,11 +7198,11 @@
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>Анализ реакции срыва 13C(d,t)12C в области энергий 13–18 мэв: определение асимптотических нормировочных коэффициентов и структуры состояний ядра 12C</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
+          <t>Анализ реакции срыва ¹³C(d,t)¹²C в области энергий 13–18 мэв: определение асимптотических нормировочных коэффициентов и структуры состояний ядра ¹²C</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="275.5" customHeight="1">
       <c r="A70" t="inlineStr">
         <is>
           <t>S2-03</t>
@@ -7253,11 +7243,11 @@
       </c>
       <c r="I70" s="4" t="inlineStr">
         <is>
-          <t>Полный и парциальные астрофизические S-факторы реакции 3He(d, p)4He в микроскопическом кластерном подходе</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
+          <t>Полный и парциальные астрофизические S-факторы реакции ³He(d, p)⁴He в микроскопическом кластерном подходе</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="72.5" customHeight="1">
       <c r="A71" t="inlineStr">
         <is>
           <t>S2-04</t>
@@ -7302,7 +7292,7 @@
         </is>
       </c>
     </row>
-    <row r="72">
+    <row r="72" ht="130.5" customHeight="1">
       <c r="A72" t="inlineStr">
         <is>
           <t>S2-05</t>
@@ -7338,11 +7328,11 @@
       </c>
       <c r="I72" s="4" t="inlineStr">
         <is>
-          <t>Multinucleon transfer reactions in 7Li, 12C,40Ar, 40,48Ca + 197Au</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
+          <t>Multinucleon transfer reactions in ⁷Li, ¹²C,⁴⁰Ar, ⁴⁰⸴ ⁴⁸Ca + ¹⁹⁷Au</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="232" customHeight="1">
       <c r="A73" t="inlineStr">
         <is>
           <t>S2-06</t>
@@ -7387,7 +7377,7 @@
         </is>
       </c>
     </row>
-    <row r="74">
+    <row r="74" ht="203" customHeight="1">
       <c r="A74" t="inlineStr">
         <is>
           <t>S2-07</t>
@@ -7432,7 +7422,7 @@
         </is>
       </c>
     </row>
-    <row r="75">
+    <row r="75" ht="203" customHeight="1">
       <c r="A75" t="inlineStr">
         <is>
           <t>S2-08</t>
@@ -7477,7 +7467,7 @@
         </is>
       </c>
     </row>
-    <row r="76">
+    <row r="76" ht="203" customHeight="1">
       <c r="A76" t="inlineStr">
         <is>
           <t>S2-09</t>
@@ -7527,7 +7517,7 @@
         </is>
       </c>
     </row>
-    <row r="77">
+    <row r="77" ht="217.5" customHeight="1">
       <c r="A77" t="inlineStr">
         <is>
           <t>S2-10</t>
@@ -7567,7 +7557,7 @@
         </is>
       </c>
     </row>
-    <row r="78">
+    <row r="78" ht="174" customHeight="1">
       <c r="A78" t="inlineStr">
         <is>
           <t>S2-11</t>
@@ -7612,7 +7602,7 @@
         </is>
       </c>
     </row>
-    <row r="79">
+    <row r="79" ht="304.5" customHeight="1">
       <c r="A79" t="inlineStr">
         <is>
           <t>S2-12</t>
@@ -7657,7 +7647,7 @@
         </is>
       </c>
     </row>
-    <row r="80">
+    <row r="80" ht="261" customHeight="1">
       <c r="A80" t="inlineStr">
         <is>
           <t>S2-13</t>
@@ -7697,7 +7687,7 @@
         </is>
       </c>
     </row>
-    <row r="81">
+    <row r="81" ht="174" customHeight="1">
       <c r="A81" t="inlineStr">
         <is>
           <t>S2-14</t>
@@ -7742,7 +7732,7 @@
         </is>
       </c>
     </row>
-    <row r="82">
+    <row r="82" ht="290" customHeight="1">
       <c r="A82" t="inlineStr">
         <is>
           <t>S2-15</t>
@@ -7782,7 +7772,7 @@
         </is>
       </c>
     </row>
-    <row r="83">
+    <row r="83" ht="145" customHeight="1">
       <c r="A83" t="inlineStr">
         <is>
           <t>S2-16</t>
@@ -7827,7 +7817,7 @@
         </is>
       </c>
     </row>
-    <row r="84">
+    <row r="84" ht="145" customHeight="1">
       <c r="A84" t="inlineStr">
         <is>
           <t>S2-17</t>
@@ -7872,7 +7862,7 @@
         </is>
       </c>
     </row>
-    <row r="85">
+    <row r="85" ht="130.5" customHeight="1">
       <c r="A85" t="inlineStr">
         <is>
           <t>S2-19</t>
@@ -7913,11 +7903,11 @@
       </c>
       <c r="I85" s="4" t="inlineStr">
         <is>
-          <t>Особенности фоторасщепления изотопов рения 185,187Re</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
+          <t>Особенности фоторасщепления изотопов рения ¹⁸⁵⸴ ¹⁸⁷Re</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="203" customHeight="1">
       <c r="A86" t="inlineStr">
         <is>
           <t>S2-20</t>
@@ -7962,7 +7952,7 @@
         </is>
       </c>
     </row>
-    <row r="87">
+    <row r="87" ht="188.5" customHeight="1">
       <c r="A87" t="inlineStr">
         <is>
           <t>S2-21</t>
@@ -8007,7 +7997,7 @@
         </is>
       </c>
     </row>
-    <row r="88">
+    <row r="88" ht="130.5" customHeight="1">
       <c r="A88" t="inlineStr">
         <is>
           <t>S2-22</t>
@@ -8043,11 +8033,11 @@
       </c>
       <c r="I88" s="4" t="inlineStr">
         <is>
-          <t>Potential description of alpha+197Au elastic scattering</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
+          <t>Potential description of α+¹⁹⁷Au elastic scattering</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="290" customHeight="1">
       <c r="A89" t="inlineStr">
         <is>
           <t>S2-23</t>
@@ -8087,7 +8077,7 @@
         </is>
       </c>
     </row>
-    <row r="90">
+    <row r="90" ht="159.5" customHeight="1">
       <c r="A90" t="inlineStr">
         <is>
           <t>S2-24</t>
@@ -8123,11 +8113,11 @@
       </c>
       <c r="I90" s="4" t="inlineStr">
         <is>
-          <t>Исследование рассеяния 6He - 4He на фрагмент-сепараторе АКУЛИНА-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
+          <t>Исследование рассеяния ⁶He - ⁴He на фрагмент-сепараторе АКУЛИНА-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="145" customHeight="1">
       <c r="A91" t="inlineStr">
         <is>
           <t>S2-25</t>
@@ -8168,11 +8158,11 @@
       </c>
       <c r="I91" s="4" t="inlineStr">
         <is>
-          <t>Experimental studies of 10B(7Li, 8Li)9B transfer reaction at 58 MeV</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
+          <t>Experimental studies of ¹⁰B(⁷Li, ⁸Li)⁹B transfer reaction at 58 MeV</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="409.5" customHeight="1">
       <c r="A92" t="inlineStr">
         <is>
           <t>S2-26</t>
@@ -8213,11 +8203,11 @@
       </c>
       <c r="I92" s="4" t="inlineStr">
         <is>
-          <t>Экспериментальный поиск аномалии при снятии возбуждения ядра 8Ве* с испусканием электрон-позитронной пары в реакции взаимодействия нейтронов с энергией свыше 20 МэВ с ядром 10В</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
+          <t>Экспериментальный поиск аномалии при снятии возбуждения ядра ⁸Ве* с испусканием электрон-позитронной пары в реакции взаимодействия нейтронов с энергией свыше 20 МэВ с ядром ¹⁰В</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="232" customHeight="1">
       <c r="A93" t="inlineStr">
         <is>
           <t>S2-27</t>
@@ -8253,11 +8243,11 @@
       </c>
       <c r="I93" s="4" t="inlineStr">
         <is>
-          <t>Изучение механизмов выбивания нейтрона в реакции 9Be(7Be, 6Be)X при промежуточной энергии</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
+          <t>Изучение механизмов выбивания нейтрона в реакции ⁹Be(⁷Be, ⁶Be)X при промежуточной энергии</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="174" customHeight="1">
       <c r="A94" t="inlineStr">
         <is>
           <t>S2-28</t>
@@ -8293,11 +8283,11 @@
       </c>
       <c r="I94" s="4" t="inlineStr">
         <is>
-          <t>Измерение угловых распределений распада 7He заселяемого в реакции 6He(d,p)</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
+          <t>Измерение угловых распределений распада ⁷He заселяемого в реакции ⁶He(d,p)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="203" customHeight="1">
       <c r="A95" t="inlineStr">
         <is>
           <t>S2-29</t>
@@ -8337,7 +8327,7 @@
         </is>
       </c>
     </row>
-    <row r="96">
+    <row r="96" ht="145" customHeight="1">
       <c r="A96" t="inlineStr">
         <is>
           <t>S2-30</t>
@@ -8377,7 +8367,7 @@
         </is>
       </c>
     </row>
-    <row r="97">
+    <row r="97" ht="188.5" customHeight="1">
       <c r="A97" t="inlineStr">
         <is>
           <t>S2-31</t>
@@ -8413,11 +8403,11 @@
       </c>
       <c r="I97" s="4" t="inlineStr">
         <is>
-          <t>237Np+48Ca reaction and decay properties of 282Nh and descendant nuclei at DGFRS‑2</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
+          <t>²³⁷Np+⁴⁸Ca reaction and decay properties of ²⁸²Nh and descendant nuclei at DGFRS‑2</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="188.5" customHeight="1">
       <c r="A98" t="inlineStr">
         <is>
           <t>S2-32</t>
@@ -8457,7 +8447,7 @@
         </is>
       </c>
     </row>
-    <row r="99">
+    <row r="99" ht="246.5" customHeight="1">
       <c r="A99" t="inlineStr">
         <is>
           <t>S2-33</t>
@@ -8493,11 +8483,11 @@
       </c>
       <c r="I99" s="4" t="inlineStr">
         <is>
-          <t>Роль нейтронного избытка в механизмах передачи нуклонов в реакциях тяжелых ионов 40, 48Ca + 197Au</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
+          <t>Роль нейтронного избытка в механизмах передачи нуклонов в реакциях тяжелых ионов ⁴⁰⸴ ⁴⁸Ca + ¹⁹⁷Au</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="159.5" customHeight="1">
       <c r="A100" t="inlineStr">
         <is>
           <t>S2-34</t>
@@ -8537,7 +8527,7 @@
         </is>
       </c>
     </row>
-    <row r="101">
+    <row r="101" ht="188.5" customHeight="1">
       <c r="A101" t="inlineStr">
         <is>
           <t>S2-35</t>
@@ -8582,7 +8572,7 @@
         </is>
       </c>
     </row>
-    <row r="102">
+    <row r="102" ht="290" customHeight="1">
       <c r="A102" t="inlineStr">
         <is>
           <t>S2-36</t>
@@ -8627,7 +8617,7 @@
         </is>
       </c>
     </row>
-    <row r="103">
+    <row r="103" ht="290" customHeight="1">
       <c r="A103" t="inlineStr">
         <is>
           <t>S3-01</t>
@@ -8672,7 +8662,7 @@
         </is>
       </c>
     </row>
-    <row r="104">
+    <row r="104" ht="232" customHeight="1">
       <c r="A104" t="inlineStr">
         <is>
           <t>S3-02</t>
@@ -8717,7 +8707,7 @@
         </is>
       </c>
     </row>
-    <row r="105">
+    <row r="105" ht="319" customHeight="1">
       <c r="A105" t="inlineStr">
         <is>
           <t>S3-03</t>
@@ -8762,7 +8752,7 @@
         </is>
       </c>
     </row>
-    <row r="106">
+    <row r="106" ht="333.5" customHeight="1">
       <c r="A106" t="inlineStr">
         <is>
           <t>S3-04</t>
@@ -8802,7 +8792,7 @@
         </is>
       </c>
     </row>
-    <row r="107">
+    <row r="107" ht="145" customHeight="1">
       <c r="A107" t="inlineStr">
         <is>
           <t>S3-05</t>
@@ -8847,7 +8837,7 @@
         </is>
       </c>
     </row>
-    <row r="108">
+    <row r="108" ht="246.5" customHeight="1">
       <c r="A108" t="inlineStr">
         <is>
           <t>S3-06</t>
@@ -8887,7 +8877,7 @@
         </is>
       </c>
     </row>
-    <row r="109">
+    <row r="109" ht="145" customHeight="1">
       <c r="A109" t="inlineStr">
         <is>
           <t>S3-07</t>
@@ -8932,7 +8922,7 @@
         </is>
       </c>
     </row>
-    <row r="110">
+    <row r="110" ht="275.5" customHeight="1">
       <c r="A110" t="inlineStr">
         <is>
           <t>S3-08</t>
@@ -8977,7 +8967,7 @@
         </is>
       </c>
     </row>
-    <row r="111">
+    <row r="111" ht="188.5" customHeight="1">
       <c r="A111" t="inlineStr">
         <is>
           <t>S3-09</t>
@@ -9017,7 +9007,7 @@
         </is>
       </c>
     </row>
-    <row r="112">
+    <row r="112" ht="116" customHeight="1">
       <c r="A112" t="inlineStr">
         <is>
           <t>S3-10</t>
@@ -9062,7 +9052,7 @@
         </is>
       </c>
     </row>
-    <row r="113">
+    <row r="113" ht="246.5" customHeight="1">
       <c r="A113" t="inlineStr">
         <is>
           <t>S3-11</t>
@@ -9107,7 +9097,7 @@
         </is>
       </c>
     </row>
-    <row r="114">
+    <row r="114" ht="188.5" customHeight="1">
       <c r="A114" t="inlineStr">
         <is>
           <t>S3-12</t>
@@ -9147,7 +9137,7 @@
         </is>
       </c>
     </row>
-    <row r="115">
+    <row r="115" ht="333.5" customHeight="1">
       <c r="A115" t="inlineStr">
         <is>
           <t>S3-13</t>
@@ -9192,7 +9182,7 @@
         </is>
       </c>
     </row>
-    <row r="116">
+    <row r="116" ht="203" customHeight="1">
       <c r="A116" t="inlineStr">
         <is>
           <t>S3-14</t>
@@ -9237,7 +9227,7 @@
         </is>
       </c>
     </row>
-    <row r="117">
+    <row r="117" ht="130.5" customHeight="1">
       <c r="A117" t="inlineStr">
         <is>
           <t>S3-15</t>
@@ -9277,7 +9267,7 @@
         </is>
       </c>
     </row>
-    <row r="118">
+    <row r="118" ht="275.5" customHeight="1">
       <c r="A118" t="inlineStr">
         <is>
           <t>S3-16</t>
@@ -9322,7 +9312,7 @@
         </is>
       </c>
     </row>
-    <row r="119">
+    <row r="119" ht="203" customHeight="1">
       <c r="A119" t="inlineStr">
         <is>
           <t>S3-17</t>
@@ -9362,7 +9352,7 @@
         </is>
       </c>
     </row>
-    <row r="120">
+    <row r="120" ht="203" customHeight="1">
       <c r="A120" t="inlineStr">
         <is>
           <t>S3-18</t>
@@ -9402,7 +9392,7 @@
         </is>
       </c>
     </row>
-    <row r="121">
+    <row r="121" ht="217.5" customHeight="1">
       <c r="A121" t="inlineStr">
         <is>
           <t>S3-19</t>
@@ -9447,7 +9437,7 @@
         </is>
       </c>
     </row>
-    <row r="122">
+    <row r="122" ht="188.5" customHeight="1">
       <c r="A122" t="inlineStr">
         <is>
           <t>S3-20</t>
@@ -9492,7 +9482,7 @@
         </is>
       </c>
     </row>
-    <row r="123">
+    <row r="123" ht="174" customHeight="1">
       <c r="A123" t="inlineStr">
         <is>
           <t>S3-21</t>
@@ -9537,7 +9527,7 @@
         </is>
       </c>
     </row>
-    <row r="124">
+    <row r="124" ht="261" customHeight="1">
       <c r="A124" t="inlineStr">
         <is>
           <t>S3-22</t>
@@ -9577,7 +9567,7 @@
         </is>
       </c>
     </row>
-    <row r="125">
+    <row r="125" ht="174" customHeight="1">
       <c r="A125" t="inlineStr">
         <is>
           <t>S3-23</t>
@@ -9613,11 +9603,11 @@
       </c>
       <c r="I125" s="4" t="inlineStr">
         <is>
-          <t>Влияние 222Rn на расчёт радиоуглеродного возраста древесных углей</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
+          <t>Влияние ²²²Rn на расчёт радиоуглеродного возраста древесных углей</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="362.5" customHeight="1">
       <c r="A126" t="inlineStr">
         <is>
           <t>S3-24</t>
@@ -9662,7 +9652,7 @@
         </is>
       </c>
     </row>
-    <row r="127">
+    <row r="127" ht="145" customHeight="1">
       <c r="A127" t="inlineStr">
         <is>
           <t>S3-25</t>
@@ -9707,7 +9697,7 @@
         </is>
       </c>
     </row>
-    <row r="128">
+    <row r="128" ht="290" customHeight="1">
       <c r="A128" t="inlineStr">
         <is>
           <t>S3-26</t>
@@ -9752,7 +9742,7 @@
         </is>
       </c>
     </row>
-    <row r="129">
+    <row r="129" ht="261" customHeight="1">
       <c r="A129" t="inlineStr">
         <is>
           <t>S3-27</t>
@@ -9792,7 +9782,7 @@
         </is>
       </c>
     </row>
-    <row r="130">
+    <row r="130" ht="232" customHeight="1">
       <c r="A130" t="inlineStr">
         <is>
           <t>S4-01</t>
@@ -9837,7 +9827,7 @@
         </is>
       </c>
     </row>
-    <row r="131">
+    <row r="131" ht="275.5" customHeight="1">
       <c r="A131" t="inlineStr">
         <is>
           <t>S4-02</t>
@@ -9882,7 +9872,7 @@
         </is>
       </c>
     </row>
-    <row r="132">
+    <row r="132" ht="130.5" customHeight="1">
       <c r="A132" t="inlineStr">
         <is>
           <t>S4-03</t>
@@ -9918,11 +9908,11 @@
       </c>
       <c r="I132" s="4" t="inlineStr">
         <is>
-          <t>Inclusive $J/\psi$ Production as a Probe of Gluon Dynamics at NICA</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
+          <t>Inclusive J/ψ Production as a Probe of Gluon Dynamics at NICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="246.5" customHeight="1">
       <c r="A133" t="inlineStr">
         <is>
           <t>S4-04</t>
@@ -9967,7 +9957,7 @@
         </is>
       </c>
     </row>
-    <row r="134">
+    <row r="134" ht="217.5" customHeight="1">
       <c r="A134" t="inlineStr">
         <is>
           <t>S4-05</t>
@@ -10012,7 +10002,7 @@
         </is>
       </c>
     </row>
-    <row r="135">
+    <row r="135" ht="188.5" customHeight="1">
       <c r="A135" t="inlineStr">
         <is>
           <t>S4-06</t>
@@ -10057,7 +10047,7 @@
         </is>
       </c>
     </row>
-    <row r="136">
+    <row r="136" ht="246.5" customHeight="1">
       <c r="A136" t="inlineStr">
         <is>
           <t>S4-07</t>
@@ -10102,7 +10092,7 @@
         </is>
       </c>
     </row>
-    <row r="137">
+    <row r="137" ht="174" customHeight="1">
       <c r="A137" t="inlineStr">
         <is>
           <t>S4-08</t>
@@ -10147,7 +10137,7 @@
         </is>
       </c>
     </row>
-    <row r="138">
+    <row r="138" ht="246.5" customHeight="1">
       <c r="A138" t="inlineStr">
         <is>
           <t>S4-09</t>
@@ -10192,7 +10182,7 @@
         </is>
       </c>
     </row>
-    <row r="139">
+    <row r="139" ht="174" customHeight="1">
       <c r="A139" t="inlineStr">
         <is>
           <t>S4-10</t>
@@ -10237,7 +10227,7 @@
         </is>
       </c>
     </row>
-    <row r="140">
+    <row r="140" ht="145" customHeight="1">
       <c r="A140" t="inlineStr">
         <is>
           <t>S4-11</t>
@@ -10278,11 +10268,11 @@
       </c>
       <c r="I140" s="4" t="inlineStr">
         <is>
-          <t>Ядро 8Be и состояние Хойла в диссоциации релятивистских ядер</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
+          <t>Ядро ⁸Be и состояние Хойла в диссоциации релятивистских ядер</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="145" customHeight="1">
       <c r="A141" t="inlineStr">
         <is>
           <t>S4-12</t>
@@ -10327,7 +10317,7 @@
         </is>
       </c>
     </row>
-    <row r="142">
+    <row r="142" ht="174" customHeight="1">
       <c r="A142" t="inlineStr">
         <is>
           <t>S4-13</t>
@@ -10372,7 +10362,7 @@
         </is>
       </c>
     </row>
-    <row r="143">
+    <row r="143" ht="232" customHeight="1">
       <c r="A143" t="inlineStr">
         <is>
           <t>S4-14</t>
@@ -10417,7 +10407,7 @@
         </is>
       </c>
     </row>
-    <row r="144">
+    <row r="144" ht="159.5" customHeight="1">
       <c r="A144" t="inlineStr">
         <is>
           <t>S4-15</t>
@@ -10462,7 +10452,7 @@
         </is>
       </c>
     </row>
-    <row r="145">
+    <row r="145" ht="246.5" customHeight="1">
       <c r="A145" t="inlineStr">
         <is>
           <t>S4-16</t>
@@ -10507,7 +10497,7 @@
         </is>
       </c>
     </row>
-    <row r="146">
+    <row r="146" ht="203" customHeight="1">
       <c r="A146" t="inlineStr">
         <is>
           <t>S4-17</t>
@@ -10552,7 +10542,7 @@
         </is>
       </c>
     </row>
-    <row r="147">
+    <row r="147" ht="319" customHeight="1">
       <c r="A147" t="inlineStr">
         <is>
           <t>S4-18</t>
@@ -10597,7 +10587,7 @@
         </is>
       </c>
     </row>
-    <row r="148">
+    <row r="148" ht="130.5" customHeight="1">
       <c r="A148" t="inlineStr">
         <is>
           <t>S4-19</t>
@@ -10637,7 +10627,7 @@
         </is>
       </c>
     </row>
-    <row r="149">
+    <row r="149" ht="72.5" customHeight="1">
       <c r="A149" t="inlineStr">
         <is>
           <t>S4-20</t>
@@ -10682,7 +10672,7 @@
         </is>
       </c>
     </row>
-    <row r="150">
+    <row r="150" ht="348" customHeight="1">
       <c r="A150" t="inlineStr">
         <is>
           <t>S4-21</t>
@@ -10727,7 +10717,7 @@
         </is>
       </c>
     </row>
-    <row r="151">
+    <row r="151" ht="319" customHeight="1">
       <c r="A151" t="inlineStr">
         <is>
           <t>S4-22</t>
@@ -10772,7 +10762,7 @@
         </is>
       </c>
     </row>
-    <row r="152">
+    <row r="152" ht="290" customHeight="1">
       <c r="A152" t="inlineStr">
         <is>
           <t>S4-23</t>
@@ -10817,7 +10807,7 @@
         </is>
       </c>
     </row>
-    <row r="153">
+    <row r="153" ht="246.5" customHeight="1">
       <c r="A153" t="inlineStr">
         <is>
           <t>S4-24</t>
@@ -10862,7 +10852,7 @@
         </is>
       </c>
     </row>
-    <row r="154">
+    <row r="154" ht="261" customHeight="1">
       <c r="A154" t="inlineStr">
         <is>
           <t>S4-25</t>
@@ -10907,7 +10897,7 @@
         </is>
       </c>
     </row>
-    <row r="155">
+    <row r="155" ht="261" customHeight="1">
       <c r="A155" t="inlineStr">
         <is>
           <t>S4-26</t>
@@ -10952,7 +10942,7 @@
         </is>
       </c>
     </row>
-    <row r="156">
+    <row r="156" ht="348" customHeight="1">
       <c r="A156" t="inlineStr">
         <is>
           <t>S4-27</t>
@@ -10988,11 +10978,11 @@
       </c>
       <c r="I156" s="4" t="inlineStr">
         <is>
-          <t>Analysis of charged and identified hadron spectra with Tsallis distributions in O+O, Kr+Kr, and Xe+Xe collisions at √sNN = 6 GeV using the UrQMD model</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
+          <t>Analysis of charged and identified hadron spectra with Tsallis distributions in O+O, Kr+Kr, and Xe+Xe collisions at √sₙₙ = 6 GeV using the UrQMD model</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="304.5" customHeight="1">
       <c r="A157" t="inlineStr">
         <is>
           <t>S4-28</t>
@@ -11033,11 +11023,11 @@
       </c>
       <c r="I157" s="4" t="inlineStr">
         <is>
-          <t>Измерение выстроенности K*-(892)-мезонов, образованных в каон-ядерных и пион-ядерных взаимодействиях на ускорительном комплексе У-70</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
+          <t>Измерение выстроенности K*⁻(892)-мезонов, образованных в каон-ядерных и пион-ядерных взаимодействиях на ускорительном комплексе У-70</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="188.5" customHeight="1">
       <c r="A158" t="inlineStr">
         <is>
           <t>S5-01</t>
@@ -11078,11 +11068,11 @@
       </c>
       <c r="I158" s="4" t="inlineStr">
         <is>
-          <t>Поиск тринейтрона в реакциях поглощения остановившихся пионов ядрами 9Be</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
+          <t>Поиск тринейтрона в реакциях поглощения остановившихся пионов ядрами ⁹Be</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="261" customHeight="1">
       <c r="A159" t="inlineStr">
         <is>
           <t>S5-02</t>
@@ -11127,7 +11117,7 @@
         </is>
       </c>
     </row>
-    <row r="160">
+    <row r="160" ht="130.5" customHeight="1">
       <c r="A160" t="inlineStr">
         <is>
           <t>S5-03</t>
@@ -11168,11 +11158,11 @@
       </c>
       <c r="I160" s="4" t="inlineStr">
         <is>
-          <t>Excited states of 6He nucleus in the SS-HORSE–NCSM approach</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
+          <t>Excited states of ⁶He nucleus in the SS-HORSE–NCSM approach</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="246.5" customHeight="1">
       <c r="A161" t="inlineStr">
         <is>
           <t>S5-04</t>
@@ -11217,7 +11207,7 @@
         </is>
       </c>
     </row>
-    <row r="162">
+    <row r="162" ht="232" customHeight="1">
       <c r="A162" t="inlineStr">
         <is>
           <t>S5-05</t>
@@ -11262,7 +11252,7 @@
         </is>
       </c>
     </row>
-    <row r="163">
+    <row r="163" ht="58" customHeight="1">
       <c r="A163" t="inlineStr">
         <is>
           <t>S5-06</t>
@@ -11302,7 +11292,7 @@
         </is>
       </c>
     </row>
-    <row r="164">
+    <row r="164" ht="130.5" customHeight="1">
       <c r="A164" t="inlineStr">
         <is>
           <t>S5-07</t>
@@ -11347,7 +11337,7 @@
         </is>
       </c>
     </row>
-    <row r="165">
+    <row r="165" ht="101.5" customHeight="1">
       <c r="A165" t="inlineStr">
         <is>
           <t>S5-08</t>
@@ -11392,7 +11382,7 @@
         </is>
       </c>
     </row>
-    <row r="166">
+    <row r="166" ht="217.5" customHeight="1">
       <c r="A166" t="inlineStr">
         <is>
           <t>S5-09</t>
@@ -11437,7 +11427,7 @@
         </is>
       </c>
     </row>
-    <row r="167">
+    <row r="167" ht="145" customHeight="1">
       <c r="A167" t="inlineStr">
         <is>
           <t>S6-01</t>
@@ -11478,11 +11468,11 @@
       </c>
       <c r="I167" s="4" t="inlineStr">
         <is>
-          <t>Поиск тяжелого стерильного нейтрино в бета-распаде 144Pr</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
+          <t>Поиск тяжелого стерильного нейтрино в бета-распаде ¹⁴⁴Pr</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="174" customHeight="1">
       <c r="A168" t="inlineStr">
         <is>
           <t>S6-02</t>
@@ -11527,7 +11517,7 @@
         </is>
       </c>
     </row>
-    <row r="169">
+    <row r="169" ht="145" customHeight="1">
       <c r="A169" t="inlineStr">
         <is>
           <t>S6-03</t>
@@ -11572,7 +11562,7 @@
         </is>
       </c>
     </row>
-    <row r="170">
+    <row r="170" ht="188.5" customHeight="1">
       <c r="A170" t="inlineStr">
         <is>
           <t>S6-04</t>
@@ -11608,11 +11598,11 @@
       </c>
       <c r="I170" s="4" t="inlineStr">
         <is>
-          <t>Search for rare processes within the GeN experiment at Kalinin nuclear power plant</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
+          <t>Search for rare processes within the νGeN experiment at Kalinin nuclear power plant</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="159.5" customHeight="1">
       <c r="A171" t="inlineStr">
         <is>
           <t>S6-05</t>
@@ -11657,7 +11647,7 @@
         </is>
       </c>
     </row>
-    <row r="172">
+    <row r="172" ht="203" customHeight="1">
       <c r="A172" t="inlineStr">
         <is>
           <t>S6-06</t>
@@ -11702,7 +11692,7 @@
         </is>
       </c>
     </row>
-    <row r="173">
+    <row r="173" ht="159.5" customHeight="1">
       <c r="A173" t="inlineStr">
         <is>
           <t>S6-07</t>
@@ -11738,11 +11728,11 @@
       </c>
       <c r="I173" s="4" t="inlineStr">
         <is>
-          <t>Analysis of radiative capture of proton 11B (p, γ) 12C at low energy</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
+          <t>Analysis of radiative capture of proton ¹¹B (p, γ) ¹²C at low energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="159.5" customHeight="1">
       <c r="A174" t="inlineStr">
         <is>
           <t>S6-08</t>
@@ -11778,11 +11768,11 @@
       </c>
       <c r="I174" s="4" t="inlineStr">
         <is>
-          <t>Characterization of the cosmic muon background in the NUGEN experiment</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
+          <t>Characterization of the cosmic muon background in the νGeN experiment</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="290" customHeight="1">
       <c r="A175" t="inlineStr">
         <is>
           <t>S7-01</t>
@@ -11822,7 +11812,7 @@
         </is>
       </c>
     </row>
-    <row r="176">
+    <row r="176" ht="232" customHeight="1">
       <c r="A176" t="inlineStr">
         <is>
           <t>S7-02</t>
@@ -11867,7 +11857,7 @@
         </is>
       </c>
     </row>
-    <row r="177">
+    <row r="177" ht="217.5" customHeight="1">
       <c r="A177" t="inlineStr">
         <is>
           <t>S7-03</t>
@@ -11908,11 +11898,11 @@
       </c>
       <c r="I177" s="4" t="inlineStr">
         <is>
-          <t>Измерение сечения реакции 12C(12C,X)11C: особенности эксперимента и оценка неопределенностей</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
+          <t>Измерение сечения реакции ¹²C(¹²C,X)¹¹C: особенности эксперимента и оценка неопределенностей</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="174" customHeight="1">
       <c r="A178" t="inlineStr">
         <is>
           <t>S7-04</t>
@@ -11957,7 +11947,7 @@
         </is>
       </c>
     </row>
-    <row r="179">
+    <row r="179" ht="319" customHeight="1">
       <c r="A179" t="inlineStr">
         <is>
           <t>S7-05</t>
@@ -12002,7 +11992,7 @@
         </is>
       </c>
     </row>
-    <row r="180">
+    <row r="180" ht="319" customHeight="1">
       <c r="A180" t="inlineStr">
         <is>
           <t>S7-06</t>
@@ -12047,7 +12037,7 @@
         </is>
       </c>
     </row>
-    <row r="181">
+    <row r="181" ht="232" customHeight="1">
       <c r="A181" t="inlineStr">
         <is>
           <t>S7-07</t>
@@ -12092,7 +12082,7 @@
         </is>
       </c>
     </row>
-    <row r="182">
+    <row r="182" ht="217.5" customHeight="1">
       <c r="A182" t="inlineStr">
         <is>
           <t>S7-08</t>
@@ -12137,7 +12127,7 @@
         </is>
       </c>
     </row>
-    <row r="183">
+    <row r="183" ht="159.5" customHeight="1">
       <c r="A183" t="inlineStr">
         <is>
           <t>S7-09</t>
@@ -12182,7 +12172,7 @@
         </is>
       </c>
     </row>
-    <row r="184">
+    <row r="184" ht="174" customHeight="1">
       <c r="A184" t="inlineStr">
         <is>
           <t>S7-10</t>
@@ -12222,7 +12212,7 @@
         </is>
       </c>
     </row>
-    <row r="185">
+    <row r="185" ht="275.5" customHeight="1">
       <c r="A185" t="inlineStr">
         <is>
           <t>S7-11</t>
@@ -12267,7 +12257,7 @@
         </is>
       </c>
     </row>
-    <row r="186">
+    <row r="186" ht="203" customHeight="1">
       <c r="A186" t="inlineStr">
         <is>
           <t>S7-12</t>
@@ -12312,7 +12302,7 @@
         </is>
       </c>
     </row>
-    <row r="187">
+    <row r="187" ht="217.5" customHeight="1">
       <c r="A187" t="inlineStr">
         <is>
           <t>S7-13</t>
@@ -12352,7 +12342,7 @@
         </is>
       </c>
     </row>
-    <row r="188">
+    <row r="188" ht="232" customHeight="1">
       <c r="A188" t="inlineStr">
         <is>
           <t>S7-14</t>
@@ -12392,7 +12382,7 @@
         </is>
       </c>
     </row>
-    <row r="189">
+    <row r="189" ht="246.5" customHeight="1">
       <c r="A189" t="inlineStr">
         <is>
           <t>S7-15</t>
@@ -12437,7 +12427,7 @@
         </is>
       </c>
     </row>
-    <row r="190">
+    <row r="190" ht="304.5" customHeight="1">
       <c r="A190" t="inlineStr">
         <is>
           <t>S7-16</t>
@@ -12482,7 +12472,7 @@
         </is>
       </c>
     </row>
-    <row r="191">
+    <row r="191" ht="159.5" customHeight="1">
       <c r="A191" t="inlineStr">
         <is>
           <t>S7-17</t>
@@ -12527,7 +12517,7 @@
         </is>
       </c>
     </row>
-    <row r="192">
+    <row r="192" ht="174" customHeight="1">
       <c r="A192" t="inlineStr">
         <is>
           <t>S7-18</t>
@@ -12572,7 +12562,7 @@
         </is>
       </c>
     </row>
-    <row r="193">
+    <row r="193" ht="261" customHeight="1">
       <c r="A193" t="inlineStr">
         <is>
           <t>S7-19</t>
@@ -12617,7 +12607,7 @@
         </is>
       </c>
     </row>
-    <row r="194">
+    <row r="194" ht="261" customHeight="1">
       <c r="A194" t="inlineStr">
         <is>
           <t>S7-20</t>
@@ -12662,7 +12652,7 @@
         </is>
       </c>
     </row>
-    <row r="195">
+    <row r="195" ht="290" customHeight="1">
       <c r="A195" t="inlineStr">
         <is>
           <t>S7-21</t>
@@ -12707,7 +12697,7 @@
         </is>
       </c>
     </row>
-    <row r="196">
+    <row r="196" ht="232" customHeight="1">
       <c r="A196" t="inlineStr">
         <is>
           <t>S7-22</t>
@@ -12752,7 +12742,7 @@
         </is>
       </c>
     </row>
-    <row r="197">
+    <row r="197" ht="174" customHeight="1">
       <c r="A197" t="inlineStr">
         <is>
           <t>S7-23</t>
@@ -12797,7 +12787,7 @@
         </is>
       </c>
     </row>
-    <row r="198">
+    <row r="198" ht="246.5" customHeight="1">
       <c r="A198" t="inlineStr">
         <is>
           <t>S7-24</t>
@@ -12859,7 +12849,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L48"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -12868,8 +12858,7 @@
     <col width="80" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="8" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -12934,7 +12923,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="188.5" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
           <t>POST-01</t>
@@ -12966,7 +12955,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="101.5" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>POST-02</t>
@@ -12998,7 +12987,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="101.5" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
           <t>POST-03</t>
@@ -13030,7 +13019,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="130.5" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>POST-04</t>
@@ -13062,7 +13051,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="87" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
           <t>POST-05</t>
@@ -13090,7 +13079,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>О природе низколежащих состояний ядра 7Li</t>
+          <t>О природе низколежащих состояний ядра ⁷Li</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -13099,7 +13088,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="87" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>POST-06</t>
@@ -13136,7 +13125,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="203" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
           <t>POST-07</t>
@@ -13173,7 +13162,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="159.5" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>POST-08</t>
@@ -13201,7 +13190,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Измерения бета-спектра 99Тс с помощью спектрометра на основе Si(Li)-детекторов</t>
+          <t>Измерения бета-спектра ⁹⁹Тс с помощью спектрометра на основе Si(Li)-детекторов</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -13210,7 +13199,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="101.5" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
           <t>POST-09</t>
@@ -13242,7 +13231,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="101.5" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
           <t>POST-10</t>
@@ -13279,7 +13268,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="87" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
           <t>POST-11</t>
@@ -13316,7 +13305,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="261" customHeight="1">
       <c r="A13" t="inlineStr">
         <is>
           <t>POST-12</t>
@@ -13353,7 +13342,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="232" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
           <t>POST-13</t>
@@ -13400,7 +13389,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="174" customHeight="1">
       <c r="A15" t="inlineStr">
         <is>
           <t>POST-14</t>
@@ -13423,7 +13412,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Расчёт сечений образования изомера серебра 108mAg в (d,p) реакциях на ускорителе ЭГП-10</t>
+          <t>Расчёт сечений образования изомера серебра ¹⁰⁸mAg в (d,p) реакциях на ускорителе ЭГП-10</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -13432,7 +13421,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="159.5" customHeight="1">
       <c r="A16" t="inlineStr">
         <is>
           <t>POST-15</t>
@@ -13469,7 +13458,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="116" customHeight="1">
       <c r="A17" t="inlineStr">
         <is>
           <t>POST-16</t>
@@ -13497,7 +13486,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Исследование реакции n + 2H → n +n+p при энергии нейтронов 20 МэВ</t>
+          <t>Исследование реакции n + ²H → n +n+p при энергии нейтронов 20 МэВ</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -13506,7 +13495,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="145" customHeight="1">
       <c r="A18" t="inlineStr">
         <is>
           <t>POST-17</t>
@@ -13543,7 +13532,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="188.5" customHeight="1">
       <c r="A19" t="inlineStr">
         <is>
           <t>POST-18</t>
@@ -13571,7 +13560,7 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Экспериментальная установка для определения спектра энергии возбуждения ядра 10Be в реакции n + 9Be</t>
+          <t>Экспериментальная установка для определения спектра энергии возбуждения ядра ¹⁰Be в реакции n + ⁹Be</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -13580,7 +13569,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="101.5" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
           <t>POST-19</t>
@@ -13617,7 +13606,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="145" customHeight="1">
       <c r="A21" t="inlineStr">
         <is>
           <t>POST-20</t>
@@ -13649,7 +13638,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="319" customHeight="1">
       <c r="A22" t="inlineStr">
         <is>
           <t>POST-21</t>
@@ -13696,7 +13685,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="203" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
           <t>POST-22</t>
@@ -13728,7 +13717,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="290" customHeight="1">
       <c r="A24" t="inlineStr">
         <is>
           <t>POST-23</t>
@@ -13760,7 +13749,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="232" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
           <t>POST-24</t>
@@ -13797,7 +13786,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="290" customHeight="1">
       <c r="A26" t="inlineStr">
         <is>
           <t>POST-25</t>
@@ -13839,7 +13828,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="174" customHeight="1">
       <c r="A27" t="inlineStr">
         <is>
           <t>POST-26</t>
@@ -13867,7 +13856,7 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Особенности ядерных реакций с получением 99mTc на пучках протонов с энергиями до 100 МэВ</t>
+          <t>Особенности ядерных реакций с получением ⁹⁹mTc на пучках протонов с энергиями до 100 МэВ</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -13881,7 +13870,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="87" customHeight="1">
       <c r="A28" t="inlineStr">
         <is>
           <t>POST-27</t>
@@ -13913,7 +13902,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="246.5" customHeight="1">
       <c r="A29" t="inlineStr">
         <is>
           <t>POST-28</t>
@@ -13950,7 +13939,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="87" customHeight="1">
       <c r="A30" t="inlineStr">
         <is>
           <t>POST-29</t>
@@ -13987,7 +13976,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="232" customHeight="1">
       <c r="A31" t="inlineStr">
         <is>
           <t>POST-30</t>
@@ -14024,7 +14013,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="203" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
           <t>POST-31</t>
@@ -14061,7 +14050,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="203" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
           <t>POST-32</t>
@@ -14098,7 +14087,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="246.5" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
           <t>POST-33</t>
@@ -14135,7 +14124,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="290" customHeight="1">
       <c r="A35" t="inlineStr">
         <is>
           <t>POST-34</t>
@@ -14167,7 +14156,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="159.5" customHeight="1">
       <c r="A36" t="inlineStr">
         <is>
           <t>POST-35</t>
@@ -14204,7 +14193,7 @@
         </is>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="290" customHeight="1">
       <c r="A37" t="inlineStr">
         <is>
           <t>POST-36</t>
@@ -14241,7 +14230,7 @@
         </is>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="145" customHeight="1">
       <c r="A38" t="inlineStr">
         <is>
           <t>POST-37</t>
@@ -14278,7 +14267,7 @@
         </is>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="217.5" customHeight="1">
       <c r="A39" t="inlineStr">
         <is>
           <t>POST-38</t>
@@ -14315,7 +14304,7 @@
         </is>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="174" customHeight="1">
       <c r="A40" t="inlineStr">
         <is>
           <t>POST-39</t>
@@ -14352,7 +14341,7 @@
         </is>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="145" customHeight="1">
       <c r="A41" t="inlineStr">
         <is>
           <t>POST-40</t>
@@ -14389,7 +14378,7 @@
         </is>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="145" customHeight="1">
       <c r="A42" t="inlineStr">
         <is>
           <t>POST-41</t>
@@ -14426,7 +14415,7 @@
         </is>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="232" customHeight="1">
       <c r="A43" t="inlineStr">
         <is>
           <t>POST-42</t>
@@ -14463,7 +14452,7 @@
         </is>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="232" customHeight="1">
       <c r="A44" t="inlineStr">
         <is>
           <t>POST-43</t>
@@ -14495,7 +14484,7 @@
         </is>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="174" customHeight="1">
       <c r="A45" t="inlineStr">
         <is>
           <t>POST-44</t>
@@ -14532,7 +14521,7 @@
         </is>
       </c>
     </row>
-    <row r="46">
+    <row r="46" ht="348" customHeight="1">
       <c r="A46" t="inlineStr">
         <is>
           <t>POST-45</t>
@@ -14564,7 +14553,7 @@
         </is>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="232" customHeight="1">
       <c r="A47" t="inlineStr">
         <is>
           <t>POST-46</t>
@@ -14596,7 +14585,7 @@
         </is>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="116" customHeight="1">
       <c r="A48" t="inlineStr">
         <is>
           <t>POST-47</t>
@@ -14650,11 +14639,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="2" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -14675,7 +14663,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="n">
+      <c r="A2" s="5" t="n">
         <v>46272.81944444445</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -14690,7 +14678,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="n">
+      <c r="A3" s="5" t="n">
         <v>46276.86666666667</v>
       </c>
       <c r="B3" t="inlineStr">

</xml_diff>